<commit_message>
fix(allocation): update lab location for SM091 to G2 Lab and SM094 to F2 Lab
</commit_message>
<xml_diff>
--- a/MECIA_HACKS_3.0_Finalist_Teams_Members.xlsx
+++ b/MECIA_HACKS_3.0_Finalist_Teams_Members.xlsx
@@ -1501,7 +1501,7 @@
         <v>MockMirror</v>
       </c>
       <c r="L31" t="str">
-        <v>F2 Lab First floor CE dept.</v>
+        <v>G2 Lab Ground floor CE dept.</v>
       </c>
     </row>
     <row r="32">
@@ -1539,7 +1539,7 @@
         <v>CertUp</v>
       </c>
       <c r="L32" t="str">
-        <v>G2 Lab Ground floor CE dept.</v>
+        <v>F2 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="33">
@@ -7106,7 +7106,7 @@
         <v>Information Technology (IT)</v>
       </c>
       <c r="K104" t="str">
-        <v>F2 Lab First floor CE dept.</v>
+        <v>G2 Lab Ground floor CE dept.</v>
       </c>
     </row>
     <row r="105">
@@ -7141,7 +7141,7 @@
         <v/>
       </c>
       <c r="K105" t="str">
-        <v>F2 Lab First floor CE dept.</v>
+        <v>G2 Lab Ground floor CE dept.</v>
       </c>
     </row>
     <row r="106">
@@ -7176,7 +7176,7 @@
         <v/>
       </c>
       <c r="K106" t="str">
-        <v>F2 Lab First floor CE dept.</v>
+        <v>G2 Lab Ground floor CE dept.</v>
       </c>
     </row>
     <row r="107">
@@ -7211,7 +7211,7 @@
         <v/>
       </c>
       <c r="K107" t="str">
-        <v>F2 Lab First floor CE dept.</v>
+        <v>G2 Lab Ground floor CE dept.</v>
       </c>
     </row>
     <row r="108">
@@ -7246,7 +7246,7 @@
         <v>Computer Science &amp; Design (CSD)</v>
       </c>
       <c r="K108" t="str">
-        <v>G2 Lab Ground floor CE dept.</v>
+        <v>F2 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="109">
@@ -7281,7 +7281,7 @@
         <v/>
       </c>
       <c r="K109" t="str">
-        <v>G2 Lab Ground floor CE dept.</v>
+        <v>F2 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="110">
@@ -7316,7 +7316,7 @@
         <v/>
       </c>
       <c r="K110" t="str">
-        <v>G2 Lab Ground floor CE dept.</v>
+        <v>F2 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="111">
@@ -7351,7 +7351,7 @@
         <v/>
       </c>
       <c r="K111" t="str">
-        <v>G2 Lab Ground floor CE dept.</v>
+        <v>F2 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="112">
@@ -11110,7 +11110,7 @@
         <v>MockMirror</v>
       </c>
       <c r="J30" t="str">
-        <v>F2 Lab First floor CE dept.</v>
+        <v>G2 Lab Ground floor CE dept.</v>
       </c>
     </row>
     <row r="31">
@@ -11142,7 +11142,7 @@
         <v>CertUp</v>
       </c>
       <c r="J31" t="str">
-        <v>G2 Lab Ground floor CE dept.</v>
+        <v>F2 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="32">

</xml_diff>

<commit_message>
feat(finalists): add team SM065 (A.S.T.R.A) as unassigned finalist for manual panel allocation
</commit_message>
<xml_diff>
--- a/MECIA_HACKS_3.0_Finalist_Teams_Members.xlsx
+++ b/MECIA_HACKS_3.0_Finalist_Teams_Members.xlsx
@@ -5,8 +5,8 @@
   <sheets>
     <sheet name="Finalist Teams" sheetId="1" r:id="rId1"/>
     <sheet name="Clean Team &amp; Members" sheetId="2" r:id="rId2"/>
-    <sheet name="All 189 Participants" sheetId="3" r:id="rId3"/>
-    <sheet name="Software Track (30)" sheetId="4" r:id="rId4"/>
+    <sheet name="All 193 Participants" sheetId="3" r:id="rId3"/>
+    <sheet name="Software Track (31)" sheetId="4" r:id="rId4"/>
     <sheet name="Hybrid Track (15)" sheetId="5" r:id="rId5"/>
     <sheet name="Hardware Track (4)" sheetId="6" r:id="rId6"/>
   </sheets>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L54"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -425,10 +425,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>TOTAL FINALIST TEAMS: 49</v>
+        <v>TOTAL FINALIST TEAMS: 50</v>
       </c>
       <c r="B2" t="str">
-        <v>SOFTWARE: 30</v>
+        <v>SOFTWARE: 31</v>
       </c>
       <c r="C2" t="str">
         <v>HYBRID: 15</v>
@@ -437,7 +437,7 @@
         <v>HARDWARE: 4</v>
       </c>
       <c r="E2" t="str">
-        <v>TOTAL PARTICIPANTS: 189</v>
+        <v>TOTAL PARTICIPANTS: 193</v>
       </c>
     </row>
     <row r="4">
@@ -1623,37 +1623,37 @@
         <v>31</v>
       </c>
       <c r="B35" t="str">
-        <v>HM016</v>
+        <v>SM065</v>
       </c>
       <c r="C35" t="str">
-        <v>TECH-♾️</v>
+        <v>A.S.T.R.A</v>
       </c>
       <c r="D35" t="str">
-        <v>Hybrid</v>
+        <v>Software</v>
       </c>
       <c r="E35" t="str">
-        <v>RUTANSHU SHAH</v>
+        <v>Aryan Mohite</v>
       </c>
       <c r="F35" t="str">
-        <v>Rudhra Nikulbhai Patel, Maitri Brahmbhatt, PARMAR BHAVYA YOGESHKUMAR</v>
+        <v>Aditya Mathur, Anshul Chainani, Ishit Bhavsar</v>
       </c>
       <c r="G35" t="str">
-        <v>Rudhra Nikulbhai Patel</v>
+        <v>Aditya Mathur</v>
       </c>
       <c r="H35" t="str">
-        <v>Maitri Brahmbhatt</v>
+        <v>Anshul Chainani</v>
       </c>
       <c r="I35" t="str">
-        <v>PARMAR BHAVYA YOGESHKUMAR</v>
+        <v>Ishit Bhavsar</v>
       </c>
       <c r="J35">
         <v>4</v>
       </c>
       <c r="K35" t="str">
-        <v>VoltSync</v>
+        <v>S.A.D.H.A.K</v>
       </c>
       <c r="L35" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="36">
@@ -1661,37 +1661,37 @@
         <v>32</v>
       </c>
       <c r="B36" t="str">
-        <v>MX031</v>
+        <v>HM016</v>
       </c>
       <c r="C36" t="str">
-        <v>Robustors</v>
+        <v>TECH-♾️</v>
       </c>
       <c r="D36" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E36" t="str">
-        <v>Maitra Parmar</v>
+        <v>RUTANSHU SHAH</v>
       </c>
       <c r="F36" t="str">
-        <v>Bhargav, Arjit Sinh Chauhan</v>
+        <v>Rudhra Nikulbhai Patel, Maitri Brahmbhatt, PARMAR BHAVYA YOGESHKUMAR</v>
       </c>
       <c r="G36" t="str">
-        <v>Bhargav</v>
+        <v>Rudhra Nikulbhai Patel</v>
       </c>
       <c r="H36" t="str">
-        <v>Arjit Sinh Chauhan</v>
+        <v>Maitri Brahmbhatt</v>
       </c>
       <c r="I36" t="str">
-        <v/>
+        <v>PARMAR BHAVYA YOGESHKUMAR</v>
       </c>
       <c r="J36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K36" t="str">
-        <v>Blind Flight</v>
+        <v>VoltSync</v>
       </c>
       <c r="L36" t="str">
-        <v>F3 Lab First floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="37">
@@ -1699,37 +1699,37 @@
         <v>33</v>
       </c>
       <c r="B37" t="str">
-        <v>HM025</v>
+        <v>MX031</v>
       </c>
       <c r="C37" t="str">
-        <v>Deep Digs</v>
+        <v>Robustors</v>
       </c>
       <c r="D37" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E37" t="str">
-        <v>RUDRA JOSHI</v>
+        <v>Maitra Parmar</v>
       </c>
       <c r="F37" t="str">
-        <v>Aditya Shah, Deep Padhiyar, Meet Makvana</v>
+        <v>Bhargav, Arjit Sinh Chauhan</v>
       </c>
       <c r="G37" t="str">
-        <v>Aditya Shah</v>
+        <v>Bhargav</v>
       </c>
       <c r="H37" t="str">
-        <v>Deep Padhiyar</v>
+        <v>Arjit Sinh Chauhan</v>
       </c>
       <c r="I37" t="str">
-        <v>Meet Makvana</v>
+        <v/>
       </c>
       <c r="J37">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K37" t="str">
-        <v>Pit Risk Analysis and Notification Appratus (PRANA)</v>
+        <v>Blind Flight</v>
       </c>
       <c r="L37" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>F3 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="38">
@@ -1737,37 +1737,37 @@
         <v>34</v>
       </c>
       <c r="B38" t="str">
-        <v>HM010</v>
+        <v>HM025</v>
       </c>
       <c r="C38" t="str">
-        <v>Bridge of Voices</v>
+        <v>Deep Digs</v>
       </c>
       <c r="D38" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E38" t="str">
-        <v>Hetvi Patel</v>
+        <v>RUDRA JOSHI</v>
       </c>
       <c r="F38" t="str">
-        <v>Anjali Jayswal, Gopi Patel, Bansi Patel</v>
+        <v>Aditya Shah, Deep Padhiyar, Meet Makvana</v>
       </c>
       <c r="G38" t="str">
-        <v>Anjali Jayswal</v>
+        <v>Aditya Shah</v>
       </c>
       <c r="H38" t="str">
-        <v>Gopi Patel</v>
+        <v>Deep Padhiyar</v>
       </c>
       <c r="I38" t="str">
-        <v>Bansi Patel</v>
+        <v>Meet Makvana</v>
       </c>
       <c r="J38">
         <v>4</v>
       </c>
       <c r="K38" t="str">
-        <v>Bridge of Voices – Smart Glove</v>
+        <v>Pit Risk Analysis and Notification Appratus (PRANA)</v>
       </c>
       <c r="L38" t="str">
-        <v>F6 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="39">
@@ -1775,37 +1775,37 @@
         <v>35</v>
       </c>
       <c r="B39" t="str">
-        <v>HM004</v>
+        <v>HM010</v>
       </c>
       <c r="C39" t="str">
-        <v>VoltVision</v>
+        <v>Bridge of Voices</v>
       </c>
       <c r="D39" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E39" t="str">
-        <v>Lakshyaa gaurang shah</v>
+        <v>Hetvi Patel</v>
       </c>
       <c r="F39" t="str">
-        <v>Taksha Adhyaru, Aatman joshi, vinay nambiar</v>
+        <v>Anjali Jayswal, Gopi Patel, Bansi Patel</v>
       </c>
       <c r="G39" t="str">
-        <v>Taksha Adhyaru</v>
+        <v>Anjali Jayswal</v>
       </c>
       <c r="H39" t="str">
-        <v>Aatman joshi</v>
+        <v>Gopi Patel</v>
       </c>
       <c r="I39" t="str">
-        <v>vinay nambiar</v>
+        <v>Bansi Patel</v>
       </c>
       <c r="J39">
         <v>4</v>
       </c>
       <c r="K39" t="str">
-        <v>smart class energy management system</v>
+        <v>Bridge of Voices – Smart Glove</v>
       </c>
       <c r="L39" t="str">
-        <v>S3 Lab Second floor CE dept.</v>
+        <v>F6 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="40">
@@ -1813,37 +1813,37 @@
         <v>36</v>
       </c>
       <c r="B40" t="str">
-        <v>HM012</v>
+        <v>HM004</v>
       </c>
       <c r="C40" t="str">
-        <v>Mech Innovators</v>
+        <v>VoltVision</v>
       </c>
       <c r="D40" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E40" t="str">
-        <v>Swayam Shah</v>
+        <v>Lakshyaa gaurang shah</v>
       </c>
       <c r="F40" t="str">
-        <v>Dharmik Sanathara, Milan Vanzara, Pursharth Singh</v>
+        <v>Taksha Adhyaru, Aatman joshi, vinay nambiar</v>
       </c>
       <c r="G40" t="str">
-        <v>Dharmik Sanathara</v>
+        <v>Taksha Adhyaru</v>
       </c>
       <c r="H40" t="str">
-        <v>Milan Vanzara</v>
+        <v>Aatman joshi</v>
       </c>
       <c r="I40" t="str">
-        <v>Pursharth Singh</v>
+        <v>vinay nambiar</v>
       </c>
       <c r="J40">
         <v>4</v>
       </c>
       <c r="K40" t="str">
-        <v>Ecobin</v>
+        <v>smart class energy management system</v>
       </c>
       <c r="L40" t="str">
-        <v>F1 Lab First floor CE dept.</v>
+        <v>S3 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="41">
@@ -1851,37 +1851,37 @@
         <v>37</v>
       </c>
       <c r="B41" t="str">
-        <v>HM013</v>
+        <v>HM012</v>
       </c>
       <c r="C41" t="str">
-        <v>Agrisense</v>
+        <v>Mech Innovators</v>
       </c>
       <c r="D41" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E41" t="str">
-        <v>CHAITANYA GIRI</v>
+        <v>Swayam Shah</v>
       </c>
       <c r="F41" t="str">
-        <v>Aarsh Patel, Hetanshi Suthar, Parth Bhatti</v>
+        <v>Dharmik Sanathara, Milan Vanzara, Pursharth Singh</v>
       </c>
       <c r="G41" t="str">
-        <v>Aarsh Patel</v>
+        <v>Dharmik Sanathara</v>
       </c>
       <c r="H41" t="str">
-        <v>Hetanshi Suthar</v>
+        <v>Milan Vanzara</v>
       </c>
       <c r="I41" t="str">
-        <v>Parth Bhatti</v>
+        <v>Pursharth Singh</v>
       </c>
       <c r="J41">
         <v>4</v>
       </c>
       <c r="K41" t="str">
-        <v>Agrisense</v>
+        <v>Ecobin</v>
       </c>
       <c r="L41" t="str">
-        <v>G3 Lab Ground floor CE dept.</v>
+        <v>F1 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="42">
@@ -1889,37 +1889,37 @@
         <v>38</v>
       </c>
       <c r="B42" t="str">
-        <v>HM008</v>
+        <v>HM013</v>
       </c>
       <c r="C42" t="str">
-        <v>Waveminds</v>
+        <v>Agrisense</v>
       </c>
       <c r="D42" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E42" t="str">
-        <v>Aryan Shah</v>
+        <v>CHAITANYA GIRI</v>
       </c>
       <c r="F42" t="str">
-        <v>Aarav Shah, Santanu Khanra, Parv Baxi</v>
+        <v>Aarsh Patel, Hetanshi Suthar, Parth Bhatti</v>
       </c>
       <c r="G42" t="str">
-        <v>Aarav Shah</v>
+        <v>Aarsh Patel</v>
       </c>
       <c r="H42" t="str">
-        <v>Santanu Khanra</v>
+        <v>Hetanshi Suthar</v>
       </c>
       <c r="I42" t="str">
-        <v>Parv Baxi</v>
+        <v>Parth Bhatti</v>
       </c>
       <c r="J42">
         <v>4</v>
       </c>
       <c r="K42" t="str">
-        <v>RF VISION</v>
+        <v>Agrisense</v>
       </c>
       <c r="L42" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>G3 Lab Ground floor CE dept.</v>
       </c>
     </row>
     <row r="43">
@@ -1927,34 +1927,34 @@
         <v>39</v>
       </c>
       <c r="B43" t="str">
-        <v>HM006</v>
+        <v>HM008</v>
       </c>
       <c r="C43" t="str">
-        <v>AeroMorph</v>
+        <v>Waveminds</v>
       </c>
       <c r="D43" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E43" t="str">
-        <v>Jadav Anvi</v>
+        <v>Aryan Shah</v>
       </c>
       <c r="F43" t="str">
-        <v>Tisha Pandya, Raj Bhanushali, Ajaya Mishra</v>
+        <v>Aarav Shah, Santanu Khanra, Parv Baxi</v>
       </c>
       <c r="G43" t="str">
-        <v>Tisha Pandya</v>
+        <v>Aarav Shah</v>
       </c>
       <c r="H43" t="str">
-        <v>Raj Bhanushali</v>
+        <v>Santanu Khanra</v>
       </c>
       <c r="I43" t="str">
-        <v>Ajaya Mishra</v>
+        <v>Parv Baxi</v>
       </c>
       <c r="J43">
         <v>4</v>
       </c>
       <c r="K43" t="str">
-        <v>Morphing Wing</v>
+        <v>RF VISION</v>
       </c>
       <c r="L43" t="str">
         <v>F5 Lab First floor CE dept.</v>
@@ -1965,37 +1965,37 @@
         <v>40</v>
       </c>
       <c r="B44" t="str">
-        <v>HM009</v>
+        <v>HM006</v>
       </c>
       <c r="C44" t="str">
-        <v>AgriMix Pro</v>
+        <v>AeroMorph</v>
       </c>
       <c r="D44" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E44" t="str">
-        <v>prajapati pratham</v>
+        <v>Jadav Anvi</v>
       </c>
       <c r="F44" t="str">
-        <v>Savya singh, Drasti bodana, Bhavya sharma</v>
+        <v>Tisha Pandya, Raj Bhanushali, Ajaya Mishra</v>
       </c>
       <c r="G44" t="str">
-        <v>Savya singh</v>
+        <v>Tisha Pandya</v>
       </c>
       <c r="H44" t="str">
-        <v>Drasti bodana</v>
+        <v>Raj Bhanushali</v>
       </c>
       <c r="I44" t="str">
-        <v>Bhavya sharma</v>
+        <v>Ajaya Mishra</v>
       </c>
       <c r="J44">
         <v>4</v>
       </c>
       <c r="K44" t="str">
-        <v>AgriMix1.0</v>
+        <v>Morphing Wing</v>
       </c>
       <c r="L44" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="45">
@@ -2003,37 +2003,37 @@
         <v>41</v>
       </c>
       <c r="B45" t="str">
-        <v>HM005</v>
+        <v>HM009</v>
       </c>
       <c r="C45" t="str">
-        <v>FusionSpark</v>
+        <v>AgriMix Pro</v>
       </c>
       <c r="D45" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E45" t="str">
-        <v>ISHA SHAH</v>
+        <v>prajapati pratham</v>
       </c>
       <c r="F45" t="str">
-        <v>KAVYA DAVE, ADITYA VALAND, JENIL SHINGALA</v>
+        <v>Savya singh, Drasti bodana, Bhavya sharma</v>
       </c>
       <c r="G45" t="str">
-        <v>KAVYA DAVE</v>
+        <v>Savya singh</v>
       </c>
       <c r="H45" t="str">
-        <v>ADITYA VALAND</v>
+        <v>Drasti bodana</v>
       </c>
       <c r="I45" t="str">
-        <v>JENIL SHINGALA</v>
+        <v>Bhavya sharma</v>
       </c>
       <c r="J45">
         <v>4</v>
       </c>
       <c r="K45" t="str">
-        <v>Root Vision</v>
+        <v>AgriMix1.0</v>
       </c>
       <c r="L45" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="46">
@@ -2041,37 +2041,37 @@
         <v>42</v>
       </c>
       <c r="B46" t="str">
-        <v>HM019</v>
+        <v>HM005</v>
       </c>
       <c r="C46" t="str">
-        <v>Fifty Shades Of Cache</v>
+        <v>FusionSpark</v>
       </c>
       <c r="D46" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E46" t="str">
-        <v>Agneloze Williams</v>
+        <v>ISHA SHAH</v>
       </c>
       <c r="F46" t="str">
-        <v>Zinkal Gadiya, Deep Thakkar, Neev Patel</v>
+        <v>KAVYA DAVE, ADITYA VALAND, JENIL SHINGALA</v>
       </c>
       <c r="G46" t="str">
-        <v>Zinkal Gadiya</v>
+        <v>KAVYA DAVE</v>
       </c>
       <c r="H46" t="str">
-        <v>Deep Thakkar</v>
+        <v>ADITYA VALAND</v>
       </c>
       <c r="I46" t="str">
-        <v>Neev Patel</v>
+        <v>JENIL SHINGALA</v>
       </c>
       <c r="J46">
         <v>4</v>
       </c>
       <c r="K46" t="str">
-        <v>Hyperlocal Pollution Evidence Engine</v>
+        <v>Root Vision</v>
       </c>
       <c r="L46" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="47">
@@ -2079,37 +2079,37 @@
         <v>43</v>
       </c>
       <c r="B47" t="str">
-        <v>HM017</v>
+        <v>HM019</v>
       </c>
       <c r="C47" t="str">
-        <v>Sky sketchers</v>
+        <v>Fifty Shades Of Cache</v>
       </c>
       <c r="D47" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E47" t="str">
-        <v>Patel Aum Dhiren</v>
+        <v>Agneloze Williams</v>
       </c>
       <c r="F47" t="str">
-        <v>Patel Ayush Saurabh, Patel Devesh Yogesh, Undaviya Devarsh Prashant</v>
+        <v>Zinkal Gadiya, Deep Thakkar, Neev Patel</v>
       </c>
       <c r="G47" t="str">
-        <v>Patel Ayush Saurabh</v>
+        <v>Zinkal Gadiya</v>
       </c>
       <c r="H47" t="str">
-        <v>Patel Devesh Yogesh</v>
+        <v>Deep Thakkar</v>
       </c>
       <c r="I47" t="str">
-        <v>Undaviya Devarsh Prashant</v>
+        <v>Neev Patel</v>
       </c>
       <c r="J47">
         <v>4</v>
       </c>
       <c r="K47" t="str">
-        <v>Project Phantom : Visualizing Stealth Technology</v>
+        <v>Hyperlocal Pollution Evidence Engine</v>
       </c>
       <c r="L47" t="str">
-        <v>F1 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="48">
@@ -2117,37 +2117,37 @@
         <v>44</v>
       </c>
       <c r="B48" t="str">
-        <v>HM002</v>
+        <v>HM017</v>
       </c>
       <c r="C48" t="str">
-        <v>Nirmana.io</v>
+        <v>Sky sketchers</v>
       </c>
       <c r="D48" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E48" t="str">
-        <v>Aum Panchal</v>
+        <v>Patel Aum Dhiren</v>
       </c>
       <c r="F48" t="str">
-        <v>Smit Chaudhari</v>
+        <v>Patel Ayush Saurabh, Patel Devesh Yogesh, Undaviya Devarsh Prashant</v>
       </c>
       <c r="G48" t="str">
-        <v>Smit Chaudhari</v>
+        <v>Patel Ayush Saurabh</v>
       </c>
       <c r="H48" t="str">
-        <v/>
+        <v>Patel Devesh Yogesh</v>
       </c>
       <c r="I48" t="str">
-        <v/>
+        <v>Undaviya Devarsh Prashant</v>
       </c>
       <c r="J48">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K48" t="str">
-        <v>GuardianPod</v>
+        <v>Project Phantom : Visualizing Stealth Technology</v>
       </c>
       <c r="L48" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>F1 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="49">
@@ -2155,37 +2155,37 @@
         <v>45</v>
       </c>
       <c r="B49" t="str">
-        <v>HM001</v>
+        <v>HM002</v>
       </c>
       <c r="C49" t="str">
-        <v>Helios</v>
+        <v>Nirmana.io</v>
       </c>
       <c r="D49" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E49" t="str">
-        <v>Jinal Bhavin Mistry</v>
+        <v>Aum Panchal</v>
       </c>
       <c r="F49" t="str">
-        <v>Rishabh Bhagchandani, Marmik Gandhi, Krishna Thorat</v>
+        <v>Smit Chaudhari</v>
       </c>
       <c r="G49" t="str">
-        <v>Rishabh Bhagchandani</v>
+        <v>Smit Chaudhari</v>
       </c>
       <c r="H49" t="str">
-        <v>Marmik Gandhi</v>
+        <v/>
       </c>
       <c r="I49" t="str">
-        <v>Krishna Thorat</v>
+        <v/>
       </c>
       <c r="J49">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K49" t="str">
-        <v>Rootwatch</v>
+        <v>GuardianPod</v>
       </c>
       <c r="L49" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="50">
@@ -2193,37 +2193,37 @@
         <v>46</v>
       </c>
       <c r="B50" t="str">
-        <v>XM004</v>
+        <v>HM001</v>
       </c>
       <c r="C50" t="str">
-        <v>FUTURESTACK</v>
+        <v>Helios</v>
       </c>
       <c r="D50" t="str">
-        <v>Hardware</v>
+        <v>Hybrid</v>
       </c>
       <c r="E50" t="str">
-        <v>PARTH N PRAJAPATI</v>
+        <v>Jinal Bhavin Mistry</v>
       </c>
       <c r="F50" t="str">
-        <v>MUDRA V CHAUHAN, HARSHIL PANCHAL, HARDEEP BHAVSAR</v>
+        <v>Rishabh Bhagchandani, Marmik Gandhi, Krishna Thorat</v>
       </c>
       <c r="G50" t="str">
-        <v>MUDRA V CHAUHAN</v>
+        <v>Rishabh Bhagchandani</v>
       </c>
       <c r="H50" t="str">
-        <v>HARSHIL PANCHAL</v>
+        <v>Marmik Gandhi</v>
       </c>
       <c r="I50" t="str">
-        <v>HARDEEP BHAVSAR</v>
+        <v>Krishna Thorat</v>
       </c>
       <c r="J50">
         <v>4</v>
       </c>
       <c r="K50" t="str">
-        <v>Natural cooling – Smart Passive Evaporative Cooling System</v>
+        <v>Rootwatch</v>
       </c>
       <c r="L50" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="51">
@@ -2231,37 +2231,37 @@
         <v>47</v>
       </c>
       <c r="B51" t="str">
-        <v>XM001</v>
+        <v>XM004</v>
       </c>
       <c r="C51" t="str">
-        <v>NextLift</v>
+        <v>FUTURESTACK</v>
       </c>
       <c r="D51" t="str">
         <v>Hardware</v>
       </c>
       <c r="E51" t="str">
-        <v>Shah Prayag Bhaveshbhai</v>
+        <v>PARTH N PRAJAPATI</v>
       </c>
       <c r="F51" t="str">
-        <v>Solanki Mudra Vishalkumar, Vasava Hetvi Subhashbhai, Patel Vishva Nileshkumar</v>
+        <v>MUDRA V CHAUHAN, HARSHIL PANCHAL, HARDEEP BHAVSAR</v>
       </c>
       <c r="G51" t="str">
-        <v>Solanki Mudra Vishalkumar</v>
+        <v>MUDRA V CHAUHAN</v>
       </c>
       <c r="H51" t="str">
-        <v>Vasava Hetvi Subhashbhai</v>
+        <v>HARSHIL PANCHAL</v>
       </c>
       <c r="I51" t="str">
-        <v>Patel Vishva Nileshkumar</v>
+        <v>HARDEEP BHAVSAR</v>
       </c>
       <c r="J51">
         <v>4</v>
       </c>
       <c r="K51" t="str">
-        <v>Ionic Wind Thruster</v>
+        <v>Natural cooling – Smart Passive Evaporative Cooling System</v>
       </c>
       <c r="L51" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="52">
@@ -2269,37 +2269,37 @@
         <v>48</v>
       </c>
       <c r="B52" t="str">
-        <v>XM005</v>
+        <v>XM001</v>
       </c>
       <c r="C52" t="str">
-        <v>VoltForage</v>
+        <v>NextLift</v>
       </c>
       <c r="D52" t="str">
         <v>Hardware</v>
       </c>
       <c r="E52" t="str">
-        <v>Shubh Prajapati</v>
+        <v>Shah Prayag Bhaveshbhai</v>
       </c>
       <c r="F52" t="str">
-        <v>Tejas Soni, Vraj Prajapati, Vaishnavi S</v>
+        <v>Solanki Mudra Vishalkumar, Vasava Hetvi Subhashbhai, Patel Vishva Nileshkumar</v>
       </c>
       <c r="G52" t="str">
-        <v>Tejas Soni</v>
+        <v>Solanki Mudra Vishalkumar</v>
       </c>
       <c r="H52" t="str">
-        <v>Vraj Prajapati</v>
+        <v>Vasava Hetvi Subhashbhai</v>
       </c>
       <c r="I52" t="str">
-        <v>Vaishnavi S</v>
+        <v>Patel Vishva Nileshkumar</v>
       </c>
       <c r="J52">
         <v>4</v>
       </c>
       <c r="K52" t="str">
-        <v>Smart Machine Health Monitoring And Protection System</v>
+        <v>Ionic Wind Thruster</v>
       </c>
       <c r="L52" t="str">
-        <v>G3 Lab Ground floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="53">
@@ -2307,49 +2307,87 @@
         <v>49</v>
       </c>
       <c r="B53" t="str">
-        <v>XM002</v>
+        <v>XM005</v>
       </c>
       <c r="C53" t="str">
-        <v>Akatsuki</v>
+        <v>VoltForage</v>
       </c>
       <c r="D53" t="str">
         <v>Hardware</v>
       </c>
       <c r="E53" t="str">
-        <v>Harnish Yogesh More</v>
+        <v>Shubh Prajapati</v>
       </c>
       <c r="F53" t="str">
-        <v>Tirth Parmar, Aditya Soni, Viraj Kalekar</v>
+        <v>Tejas Soni, Vraj Prajapati, Vaishnavi S</v>
       </c>
       <c r="G53" t="str">
-        <v>Tirth Parmar</v>
+        <v>Tejas Soni</v>
       </c>
       <c r="H53" t="str">
-        <v>Aditya Soni</v>
+        <v>Vraj Prajapati</v>
       </c>
       <c r="I53" t="str">
-        <v>Viraj Kalekar</v>
+        <v>Vaishnavi S</v>
       </c>
       <c r="J53">
         <v>4</v>
       </c>
       <c r="K53" t="str">
-        <v>Transformer Feedback System</v>
+        <v>Smart Machine Health Monitoring And Protection System</v>
       </c>
       <c r="L53" t="str">
         <v>G3 Lab Ground floor CE dept.</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54">
+        <v>50</v>
+      </c>
+      <c r="B54" t="str">
+        <v>XM002</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Akatsuki</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Hardware</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Harnish Yogesh More</v>
+      </c>
+      <c r="F54" t="str">
+        <v>Tirth Parmar, Aditya Soni, Viraj Kalekar</v>
+      </c>
+      <c r="G54" t="str">
+        <v>Tirth Parmar</v>
+      </c>
+      <c r="H54" t="str">
+        <v>Aditya Soni</v>
+      </c>
+      <c r="I54" t="str">
+        <v>Viraj Kalekar</v>
+      </c>
+      <c r="J54">
+        <v>4</v>
+      </c>
+      <c r="K54" t="str">
+        <v>Transformer Feedback System</v>
+      </c>
+      <c r="L54" t="str">
+        <v>G3 Lab Ground floor CE dept.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L54"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G51"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -3075,451 +3113,474 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>HM016</v>
+        <v>SM065</v>
       </c>
       <c r="B32" t="str">
-        <v>TECH-♾️</v>
+        <v>A.S.T.R.A</v>
       </c>
       <c r="C32" t="str">
-        <v>RUTANSHU SHAH</v>
+        <v>Aryan Mohite</v>
       </c>
       <c r="D32" t="str">
-        <v>Rudhra Nikulbhai Patel, Maitri Brahmbhatt, PARMAR BHAVYA YOGESHKUMAR</v>
+        <v>Aditya Mathur, Anshul Chainani, Ishit Bhavsar</v>
       </c>
       <c r="E32" t="str">
-        <v>Rudhra Nikulbhai Patel</v>
+        <v>Aditya Mathur</v>
       </c>
       <c r="F32" t="str">
-        <v>Maitri Brahmbhatt</v>
+        <v>Anshul Chainani</v>
       </c>
       <c r="G32" t="str">
-        <v>PARMAR BHAVYA YOGESHKUMAR</v>
+        <v>Ishit Bhavsar</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>MX031</v>
+        <v>HM016</v>
       </c>
       <c r="B33" t="str">
-        <v>Robustors</v>
+        <v>TECH-♾️</v>
       </c>
       <c r="C33" t="str">
-        <v>Maitra Parmar</v>
+        <v>RUTANSHU SHAH</v>
       </c>
       <c r="D33" t="str">
-        <v>Bhargav, Arjit Sinh Chauhan</v>
+        <v>Rudhra Nikulbhai Patel, Maitri Brahmbhatt, PARMAR BHAVYA YOGESHKUMAR</v>
       </c>
       <c r="E33" t="str">
-        <v>Bhargav</v>
+        <v>Rudhra Nikulbhai Patel</v>
       </c>
       <c r="F33" t="str">
-        <v>Arjit Sinh Chauhan</v>
+        <v>Maitri Brahmbhatt</v>
       </c>
       <c r="G33" t="str">
-        <v/>
+        <v>PARMAR BHAVYA YOGESHKUMAR</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>HM025</v>
+        <v>MX031</v>
       </c>
       <c r="B34" t="str">
-        <v>Deep Digs</v>
+        <v>Robustors</v>
       </c>
       <c r="C34" t="str">
-        <v>RUDRA JOSHI</v>
+        <v>Maitra Parmar</v>
       </c>
       <c r="D34" t="str">
-        <v>Aditya Shah, Deep Padhiyar, Meet Makvana</v>
+        <v>Bhargav, Arjit Sinh Chauhan</v>
       </c>
       <c r="E34" t="str">
-        <v>Aditya Shah</v>
+        <v>Bhargav</v>
       </c>
       <c r="F34" t="str">
-        <v>Deep Padhiyar</v>
+        <v>Arjit Sinh Chauhan</v>
       </c>
       <c r="G34" t="str">
-        <v>Meet Makvana</v>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>HM010</v>
+        <v>HM025</v>
       </c>
       <c r="B35" t="str">
-        <v>Bridge of Voices</v>
+        <v>Deep Digs</v>
       </c>
       <c r="C35" t="str">
-        <v>Hetvi Patel</v>
+        <v>RUDRA JOSHI</v>
       </c>
       <c r="D35" t="str">
-        <v>Anjali Jayswal, Gopi Patel, Bansi Patel</v>
+        <v>Aditya Shah, Deep Padhiyar, Meet Makvana</v>
       </c>
       <c r="E35" t="str">
-        <v>Anjali Jayswal</v>
+        <v>Aditya Shah</v>
       </c>
       <c r="F35" t="str">
-        <v>Gopi Patel</v>
+        <v>Deep Padhiyar</v>
       </c>
       <c r="G35" t="str">
-        <v>Bansi Patel</v>
+        <v>Meet Makvana</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>HM004</v>
+        <v>HM010</v>
       </c>
       <c r="B36" t="str">
-        <v>VoltVision</v>
+        <v>Bridge of Voices</v>
       </c>
       <c r="C36" t="str">
-        <v>Lakshyaa gaurang shah</v>
+        <v>Hetvi Patel</v>
       </c>
       <c r="D36" t="str">
-        <v>Taksha Adhyaru, Aatman joshi, vinay nambiar</v>
+        <v>Anjali Jayswal, Gopi Patel, Bansi Patel</v>
       </c>
       <c r="E36" t="str">
-        <v>Taksha Adhyaru</v>
+        <v>Anjali Jayswal</v>
       </c>
       <c r="F36" t="str">
-        <v>Aatman joshi</v>
+        <v>Gopi Patel</v>
       </c>
       <c r="G36" t="str">
-        <v>vinay nambiar</v>
+        <v>Bansi Patel</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>HM012</v>
+        <v>HM004</v>
       </c>
       <c r="B37" t="str">
-        <v>Mech Innovators</v>
+        <v>VoltVision</v>
       </c>
       <c r="C37" t="str">
-        <v>Swayam Shah</v>
+        <v>Lakshyaa gaurang shah</v>
       </c>
       <c r="D37" t="str">
-        <v>Dharmik Sanathara, Milan Vanzara, Pursharth Singh</v>
+        <v>Taksha Adhyaru, Aatman joshi, vinay nambiar</v>
       </c>
       <c r="E37" t="str">
-        <v>Dharmik Sanathara</v>
+        <v>Taksha Adhyaru</v>
       </c>
       <c r="F37" t="str">
-        <v>Milan Vanzara</v>
+        <v>Aatman joshi</v>
       </c>
       <c r="G37" t="str">
-        <v>Pursharth Singh</v>
+        <v>vinay nambiar</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>HM013</v>
+        <v>HM012</v>
       </c>
       <c r="B38" t="str">
-        <v>Agrisense</v>
+        <v>Mech Innovators</v>
       </c>
       <c r="C38" t="str">
-        <v>CHAITANYA GIRI</v>
+        <v>Swayam Shah</v>
       </c>
       <c r="D38" t="str">
-        <v>Aarsh Patel, Hetanshi Suthar, Parth Bhatti</v>
+        <v>Dharmik Sanathara, Milan Vanzara, Pursharth Singh</v>
       </c>
       <c r="E38" t="str">
-        <v>Aarsh Patel</v>
+        <v>Dharmik Sanathara</v>
       </c>
       <c r="F38" t="str">
-        <v>Hetanshi Suthar</v>
+        <v>Milan Vanzara</v>
       </c>
       <c r="G38" t="str">
-        <v>Parth Bhatti</v>
+        <v>Pursharth Singh</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>HM008</v>
+        <v>HM013</v>
       </c>
       <c r="B39" t="str">
-        <v>Waveminds</v>
+        <v>Agrisense</v>
       </c>
       <c r="C39" t="str">
-        <v>Aryan Shah</v>
+        <v>CHAITANYA GIRI</v>
       </c>
       <c r="D39" t="str">
-        <v>Aarav Shah, Santanu Khanra, Parv Baxi</v>
+        <v>Aarsh Patel, Hetanshi Suthar, Parth Bhatti</v>
       </c>
       <c r="E39" t="str">
-        <v>Aarav Shah</v>
+        <v>Aarsh Patel</v>
       </c>
       <c r="F39" t="str">
-        <v>Santanu Khanra</v>
+        <v>Hetanshi Suthar</v>
       </c>
       <c r="G39" t="str">
-        <v>Parv Baxi</v>
+        <v>Parth Bhatti</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>HM006</v>
+        <v>HM008</v>
       </c>
       <c r="B40" t="str">
-        <v>AeroMorph</v>
+        <v>Waveminds</v>
       </c>
       <c r="C40" t="str">
-        <v>Jadav Anvi</v>
+        <v>Aryan Shah</v>
       </c>
       <c r="D40" t="str">
-        <v>Tisha Pandya, Raj Bhanushali, Ajaya Mishra</v>
+        <v>Aarav Shah, Santanu Khanra, Parv Baxi</v>
       </c>
       <c r="E40" t="str">
-        <v>Tisha Pandya</v>
+        <v>Aarav Shah</v>
       </c>
       <c r="F40" t="str">
-        <v>Raj Bhanushali</v>
+        <v>Santanu Khanra</v>
       </c>
       <c r="G40" t="str">
-        <v>Ajaya Mishra</v>
+        <v>Parv Baxi</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>HM009</v>
+        <v>HM006</v>
       </c>
       <c r="B41" t="str">
-        <v>AgriMix Pro</v>
+        <v>AeroMorph</v>
       </c>
       <c r="C41" t="str">
-        <v>prajapati pratham</v>
+        <v>Jadav Anvi</v>
       </c>
       <c r="D41" t="str">
-        <v>Savya singh, Drasti bodana, Bhavya sharma</v>
+        <v>Tisha Pandya, Raj Bhanushali, Ajaya Mishra</v>
       </c>
       <c r="E41" t="str">
-        <v>Savya singh</v>
+        <v>Tisha Pandya</v>
       </c>
       <c r="F41" t="str">
-        <v>Drasti bodana</v>
+        <v>Raj Bhanushali</v>
       </c>
       <c r="G41" t="str">
-        <v>Bhavya sharma</v>
+        <v>Ajaya Mishra</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>HM005</v>
+        <v>HM009</v>
       </c>
       <c r="B42" t="str">
-        <v>FusionSpark</v>
+        <v>AgriMix Pro</v>
       </c>
       <c r="C42" t="str">
-        <v>ISHA SHAH</v>
+        <v>prajapati pratham</v>
       </c>
       <c r="D42" t="str">
-        <v>KAVYA DAVE, ADITYA VALAND, JENIL SHINGALA</v>
+        <v>Savya singh, Drasti bodana, Bhavya sharma</v>
       </c>
       <c r="E42" t="str">
-        <v>KAVYA DAVE</v>
+        <v>Savya singh</v>
       </c>
       <c r="F42" t="str">
-        <v>ADITYA VALAND</v>
+        <v>Drasti bodana</v>
       </c>
       <c r="G42" t="str">
-        <v>JENIL SHINGALA</v>
+        <v>Bhavya sharma</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>HM019</v>
+        <v>HM005</v>
       </c>
       <c r="B43" t="str">
-        <v>Fifty Shades Of Cache</v>
+        <v>FusionSpark</v>
       </c>
       <c r="C43" t="str">
-        <v>Agneloze Williams</v>
+        <v>ISHA SHAH</v>
       </c>
       <c r="D43" t="str">
-        <v>Zinkal Gadiya, Deep Thakkar, Neev Patel</v>
+        <v>KAVYA DAVE, ADITYA VALAND, JENIL SHINGALA</v>
       </c>
       <c r="E43" t="str">
-        <v>Zinkal Gadiya</v>
+        <v>KAVYA DAVE</v>
       </c>
       <c r="F43" t="str">
-        <v>Deep Thakkar</v>
+        <v>ADITYA VALAND</v>
       </c>
       <c r="G43" t="str">
-        <v>Neev Patel</v>
+        <v>JENIL SHINGALA</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>HM017</v>
+        <v>HM019</v>
       </c>
       <c r="B44" t="str">
-        <v>Sky sketchers</v>
+        <v>Fifty Shades Of Cache</v>
       </c>
       <c r="C44" t="str">
-        <v>Patel Aum Dhiren</v>
+        <v>Agneloze Williams</v>
       </c>
       <c r="D44" t="str">
-        <v>Patel Ayush Saurabh, Patel Devesh Yogesh, Undaviya Devarsh Prashant</v>
+        <v>Zinkal Gadiya, Deep Thakkar, Neev Patel</v>
       </c>
       <c r="E44" t="str">
-        <v>Patel Ayush Saurabh</v>
+        <v>Zinkal Gadiya</v>
       </c>
       <c r="F44" t="str">
-        <v>Patel Devesh Yogesh</v>
+        <v>Deep Thakkar</v>
       </c>
       <c r="G44" t="str">
-        <v>Undaviya Devarsh Prashant</v>
+        <v>Neev Patel</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>HM002</v>
+        <v>HM017</v>
       </c>
       <c r="B45" t="str">
-        <v>Nirmana.io</v>
+        <v>Sky sketchers</v>
       </c>
       <c r="C45" t="str">
-        <v>Aum Panchal</v>
+        <v>Patel Aum Dhiren</v>
       </c>
       <c r="D45" t="str">
-        <v>Smit Chaudhari</v>
+        <v>Patel Ayush Saurabh, Patel Devesh Yogesh, Undaviya Devarsh Prashant</v>
       </c>
       <c r="E45" t="str">
-        <v>Smit Chaudhari</v>
+        <v>Patel Ayush Saurabh</v>
       </c>
       <c r="F45" t="str">
-        <v/>
+        <v>Patel Devesh Yogesh</v>
       </c>
       <c r="G45" t="str">
-        <v/>
+        <v>Undaviya Devarsh Prashant</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>HM001</v>
+        <v>HM002</v>
       </c>
       <c r="B46" t="str">
-        <v>Helios</v>
+        <v>Nirmana.io</v>
       </c>
       <c r="C46" t="str">
-        <v>Jinal Bhavin Mistry</v>
+        <v>Aum Panchal</v>
       </c>
       <c r="D46" t="str">
-        <v>Rishabh Bhagchandani, Marmik Gandhi, Krishna Thorat</v>
+        <v>Smit Chaudhari</v>
       </c>
       <c r="E46" t="str">
-        <v>Rishabh Bhagchandani</v>
+        <v>Smit Chaudhari</v>
       </c>
       <c r="F46" t="str">
-        <v>Marmik Gandhi</v>
+        <v/>
       </c>
       <c r="G46" t="str">
-        <v>Krishna Thorat</v>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>XM004</v>
+        <v>HM001</v>
       </c>
       <c r="B47" t="str">
-        <v>FUTURESTACK</v>
+        <v>Helios</v>
       </c>
       <c r="C47" t="str">
-        <v>PARTH N PRAJAPATI</v>
+        <v>Jinal Bhavin Mistry</v>
       </c>
       <c r="D47" t="str">
-        <v>MUDRA V CHAUHAN, HARSHIL PANCHAL, HARDEEP BHAVSAR</v>
+        <v>Rishabh Bhagchandani, Marmik Gandhi, Krishna Thorat</v>
       </c>
       <c r="E47" t="str">
-        <v>MUDRA V CHAUHAN</v>
+        <v>Rishabh Bhagchandani</v>
       </c>
       <c r="F47" t="str">
-        <v>HARSHIL PANCHAL</v>
+        <v>Marmik Gandhi</v>
       </c>
       <c r="G47" t="str">
-        <v>HARDEEP BHAVSAR</v>
+        <v>Krishna Thorat</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>XM001</v>
+        <v>XM004</v>
       </c>
       <c r="B48" t="str">
-        <v>NextLift</v>
+        <v>FUTURESTACK</v>
       </c>
       <c r="C48" t="str">
-        <v>Shah Prayag Bhaveshbhai</v>
+        <v>PARTH N PRAJAPATI</v>
       </c>
       <c r="D48" t="str">
-        <v>Solanki Mudra Vishalkumar, Vasava Hetvi Subhashbhai, Patel Vishva Nileshkumar</v>
+        <v>MUDRA V CHAUHAN, HARSHIL PANCHAL, HARDEEP BHAVSAR</v>
       </c>
       <c r="E48" t="str">
-        <v>Solanki Mudra Vishalkumar</v>
+        <v>MUDRA V CHAUHAN</v>
       </c>
       <c r="F48" t="str">
-        <v>Vasava Hetvi Subhashbhai</v>
+        <v>HARSHIL PANCHAL</v>
       </c>
       <c r="G48" t="str">
-        <v>Patel Vishva Nileshkumar</v>
+        <v>HARDEEP BHAVSAR</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>XM005</v>
+        <v>XM001</v>
       </c>
       <c r="B49" t="str">
-        <v>VoltForage</v>
+        <v>NextLift</v>
       </c>
       <c r="C49" t="str">
-        <v>Shubh Prajapati</v>
+        <v>Shah Prayag Bhaveshbhai</v>
       </c>
       <c r="D49" t="str">
-        <v>Tejas Soni, Vraj Prajapati, Vaishnavi S</v>
+        <v>Solanki Mudra Vishalkumar, Vasava Hetvi Subhashbhai, Patel Vishva Nileshkumar</v>
       </c>
       <c r="E49" t="str">
-        <v>Tejas Soni</v>
+        <v>Solanki Mudra Vishalkumar</v>
       </c>
       <c r="F49" t="str">
-        <v>Vraj Prajapati</v>
+        <v>Vasava Hetvi Subhashbhai</v>
       </c>
       <c r="G49" t="str">
-        <v>Vaishnavi S</v>
+        <v>Patel Vishva Nileshkumar</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
+        <v>XM005</v>
+      </c>
+      <c r="B50" t="str">
+        <v>VoltForage</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Shubh Prajapati</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Tejas Soni, Vraj Prajapati, Vaishnavi S</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Tejas Soni</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Vraj Prajapati</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Vaishnavi S</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
         <v>XM002</v>
       </c>
-      <c r="B50" t="str">
+      <c r="B51" t="str">
         <v>Akatsuki</v>
       </c>
-      <c r="C50" t="str">
+      <c r="C51" t="str">
         <v>Harnish Yogesh More</v>
       </c>
-      <c r="D50" t="str">
+      <c r="D51" t="str">
         <v>Tirth Parmar, Aditya Soni, Viraj Kalekar</v>
       </c>
-      <c r="E50" t="str">
+      <c r="E51" t="str">
         <v>Tirth Parmar</v>
       </c>
-      <c r="F50" t="str">
+      <c r="F51" t="str">
         <v>Aditya Soni</v>
       </c>
-      <c r="G50" t="str">
+      <c r="G51" t="str">
         <v>Viraj Kalekar</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G51"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K192"/>
+  <dimension ref="A1:K196"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -3536,7 +3597,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>MECIA HACKS 3.0 — ALL FINALIST PARTICIPANTS ROSTER (189 PARTICIPANTS)</v>
+        <v>MECIA HACKS 3.0 — ALL FINALIST PARTICIPANTS ROSTER (193 PARTICIPANTS)</v>
       </c>
     </row>
     <row r="3">
@@ -7639,34 +7700,34 @@
         <v>117</v>
       </c>
       <c r="B120" t="str">
-        <v>HM016</v>
+        <v>SM065</v>
       </c>
       <c r="C120" t="str">
-        <v>TECH-♾️</v>
+        <v>A.S.T.R.A</v>
       </c>
       <c r="D120" t="str">
-        <v>Hybrid</v>
+        <v>Software</v>
       </c>
       <c r="E120" t="str">
         <v>Team Leader</v>
       </c>
       <c r="F120" t="str">
-        <v>RUTANSHU SHAH</v>
+        <v>Aryan Mohite</v>
       </c>
       <c r="G120" t="str">
-        <v>250410111029</v>
+        <v>250410111002</v>
       </c>
       <c r="H120" t="str">
-        <v>8238806560</v>
+        <v>7383232176</v>
       </c>
       <c r="I120" t="str">
-        <v>rutanshu001@gmail.com</v>
+        <v>aryanmohite0707@gmail.com</v>
       </c>
       <c r="J120" t="str">
         <v>Electronics &amp; Communication (EC)</v>
       </c>
       <c r="K120" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="121">
@@ -7674,25 +7735,25 @@
         <v>118</v>
       </c>
       <c r="B121" t="str">
-        <v>HM016</v>
+        <v>SM065</v>
       </c>
       <c r="C121" t="str">
-        <v>TECH-♾️</v>
+        <v>A.S.T.R.A</v>
       </c>
       <c r="D121" t="str">
-        <v>Hybrid</v>
+        <v>Software</v>
       </c>
       <c r="E121" t="str">
         <v>Member 1</v>
       </c>
       <c r="F121" t="str">
-        <v>Rudhra Nikulbhai Patel</v>
+        <v>Aditya Mathur</v>
       </c>
       <c r="G121" t="str">
-        <v>250410107131</v>
+        <v>250410107005</v>
       </c>
       <c r="H121" t="str">
-        <v>9913217394</v>
+        <v>8347068168</v>
       </c>
       <c r="I121" t="str">
         <v/>
@@ -7701,7 +7762,7 @@
         <v/>
       </c>
       <c r="K121" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="122">
@@ -7709,25 +7770,25 @@
         <v>119</v>
       </c>
       <c r="B122" t="str">
-        <v>HM016</v>
+        <v>SM065</v>
       </c>
       <c r="C122" t="str">
-        <v>TECH-♾️</v>
+        <v>A.S.T.R.A</v>
       </c>
       <c r="D122" t="str">
-        <v>Hybrid</v>
+        <v>Software</v>
       </c>
       <c r="E122" t="str">
         <v>Member 2</v>
       </c>
       <c r="F122" t="str">
-        <v>Maitri Brahmbhatt</v>
+        <v>Anshul Chainani</v>
       </c>
       <c r="G122" t="str">
-        <v>250410107019</v>
+        <v>250410107010</v>
       </c>
       <c r="H122" t="str">
-        <v>9879489218</v>
+        <v>9428173391</v>
       </c>
       <c r="I122" t="str">
         <v/>
@@ -7736,7 +7797,7 @@
         <v/>
       </c>
       <c r="K122" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="123">
@@ -7744,25 +7805,25 @@
         <v>120</v>
       </c>
       <c r="B123" t="str">
-        <v>HM016</v>
+        <v>SM065</v>
       </c>
       <c r="C123" t="str">
-        <v>TECH-♾️</v>
+        <v>A.S.T.R.A</v>
       </c>
       <c r="D123" t="str">
-        <v>Hybrid</v>
+        <v>Software</v>
       </c>
       <c r="E123" t="str">
         <v>Member 3</v>
       </c>
       <c r="F123" t="str">
-        <v>PARMAR BHAVYA YOGESHKUMAR</v>
+        <v>Ishit Bhavsar</v>
       </c>
       <c r="G123" t="str">
-        <v>250410107099</v>
+        <v>250410107018</v>
       </c>
       <c r="H123" t="str">
-        <v>7621830995</v>
+        <v>8866417323</v>
       </c>
       <c r="I123" t="str">
         <v/>
@@ -7771,7 +7832,7 @@
         <v/>
       </c>
       <c r="K123" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="124">
@@ -7779,10 +7840,10 @@
         <v>121</v>
       </c>
       <c r="B124" t="str">
-        <v>MX031</v>
+        <v>HM016</v>
       </c>
       <c r="C124" t="str">
-        <v>Robustors</v>
+        <v>TECH-♾️</v>
       </c>
       <c r="D124" t="str">
         <v>Hybrid</v>
@@ -7791,22 +7852,22 @@
         <v>Team Leader</v>
       </c>
       <c r="F124" t="str">
-        <v>Maitra Parmar</v>
+        <v>RUTANSHU SHAH</v>
       </c>
       <c r="G124" t="str">
-        <v>250410111015</v>
+        <v>250410111029</v>
       </c>
       <c r="H124" t="str">
-        <v>9409689125</v>
+        <v>8238806560</v>
       </c>
       <c r="I124" t="str">
-        <v>maitraparmar125@gmail.com</v>
+        <v>rutanshu001@gmail.com</v>
       </c>
       <c r="J124" t="str">
         <v>Electronics &amp; Communication (EC)</v>
       </c>
       <c r="K124" t="str">
-        <v>F3 Lab First floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="125">
@@ -7814,10 +7875,10 @@
         <v>122</v>
       </c>
       <c r="B125" t="str">
-        <v>MX031</v>
+        <v>HM016</v>
       </c>
       <c r="C125" t="str">
-        <v>Robustors</v>
+        <v>TECH-♾️</v>
       </c>
       <c r="D125" t="str">
         <v>Hybrid</v>
@@ -7826,13 +7887,13 @@
         <v>Member 1</v>
       </c>
       <c r="F125" t="str">
-        <v>Bhargav</v>
+        <v>Rudhra Nikulbhai Patel</v>
       </c>
       <c r="G125" t="str">
-        <v>250410116029</v>
+        <v>250410107131</v>
       </c>
       <c r="H125" t="str">
-        <v>8799092871</v>
+        <v>9913217394</v>
       </c>
       <c r="I125" t="str">
         <v/>
@@ -7841,7 +7902,7 @@
         <v/>
       </c>
       <c r="K125" t="str">
-        <v>F3 Lab First floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="126">
@@ -7849,10 +7910,10 @@
         <v>123</v>
       </c>
       <c r="B126" t="str">
-        <v>MX031</v>
+        <v>HM016</v>
       </c>
       <c r="C126" t="str">
-        <v>Robustors</v>
+        <v>TECH-♾️</v>
       </c>
       <c r="D126" t="str">
         <v>Hybrid</v>
@@ -7861,13 +7922,13 @@
         <v>Member 2</v>
       </c>
       <c r="F126" t="str">
-        <v>Arjit Sinh Chauhan</v>
+        <v>Maitri Brahmbhatt</v>
       </c>
       <c r="G126" t="str">
-        <v>250410116012</v>
+        <v>250410107019</v>
       </c>
       <c r="H126" t="str">
-        <v>8140133159</v>
+        <v>9879489218</v>
       </c>
       <c r="I126" t="str">
         <v/>
@@ -7876,7 +7937,7 @@
         <v/>
       </c>
       <c r="K126" t="str">
-        <v>F3 Lab First floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="127">
@@ -7884,34 +7945,34 @@
         <v>124</v>
       </c>
       <c r="B127" t="str">
-        <v>HM025</v>
+        <v>HM016</v>
       </c>
       <c r="C127" t="str">
-        <v>Deep Digs</v>
+        <v>TECH-♾️</v>
       </c>
       <c r="D127" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E127" t="str">
-        <v>Team Leader</v>
+        <v>Member 3</v>
       </c>
       <c r="F127" t="str">
-        <v>RUDRA JOSHI</v>
+        <v>PARMAR BHAVYA YOGESHKUMAR</v>
       </c>
       <c r="G127" t="str">
-        <v>24041011039</v>
+        <v>250410107099</v>
       </c>
       <c r="H127" t="str">
-        <v>8866052251</v>
+        <v>7621830995</v>
       </c>
       <c r="I127" t="str">
-        <v>rudraashu4@gmail.com</v>
+        <v/>
       </c>
       <c r="J127" t="str">
-        <v>Information Technology (IT)</v>
+        <v/>
       </c>
       <c r="K127" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="128">
@@ -7919,34 +7980,34 @@
         <v>125</v>
       </c>
       <c r="B128" t="str">
-        <v>HM025</v>
+        <v>MX031</v>
       </c>
       <c r="C128" t="str">
-        <v>Deep Digs</v>
+        <v>Robustors</v>
       </c>
       <c r="D128" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E128" t="str">
-        <v>Member 1</v>
+        <v>Team Leader</v>
       </c>
       <c r="F128" t="str">
-        <v>Aditya Shah</v>
+        <v>Maitra Parmar</v>
       </c>
       <c r="G128" t="str">
-        <v>240410116001</v>
+        <v>250410111015</v>
       </c>
       <c r="H128" t="str">
-        <v>8849100417</v>
+        <v>9409689125</v>
       </c>
       <c r="I128" t="str">
-        <v/>
+        <v>maitraparmar125@gmail.com</v>
       </c>
       <c r="J128" t="str">
-        <v/>
+        <v>Electronics &amp; Communication (EC)</v>
       </c>
       <c r="K128" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>F3 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="129">
@@ -7954,25 +8015,25 @@
         <v>126</v>
       </c>
       <c r="B129" t="str">
-        <v>HM025</v>
+        <v>MX031</v>
       </c>
       <c r="C129" t="str">
-        <v>Deep Digs</v>
+        <v>Robustors</v>
       </c>
       <c r="D129" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E129" t="str">
-        <v>Member 2</v>
+        <v>Member 1</v>
       </c>
       <c r="F129" t="str">
-        <v>Deep Padhiyar</v>
+        <v>Bhargav</v>
       </c>
       <c r="G129" t="str">
-        <v>240410116017</v>
+        <v>250410116029</v>
       </c>
       <c r="H129" t="str">
-        <v>9016622658</v>
+        <v>8799092871</v>
       </c>
       <c r="I129" t="str">
         <v/>
@@ -7981,7 +8042,7 @@
         <v/>
       </c>
       <c r="K129" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>F3 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="130">
@@ -7989,25 +8050,25 @@
         <v>127</v>
       </c>
       <c r="B130" t="str">
-        <v>HM025</v>
+        <v>MX031</v>
       </c>
       <c r="C130" t="str">
-        <v>Deep Digs</v>
+        <v>Robustors</v>
       </c>
       <c r="D130" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E130" t="str">
-        <v>Member 3</v>
+        <v>Member 2</v>
       </c>
       <c r="F130" t="str">
-        <v>Meet Makvana</v>
+        <v>Arjit Sinh Chauhan</v>
       </c>
       <c r="G130" t="str">
-        <v>240410116045</v>
+        <v>250410116012</v>
       </c>
       <c r="H130" t="str">
-        <v>7016808631</v>
+        <v>8140133159</v>
       </c>
       <c r="I130" t="str">
         <v/>
@@ -8016,7 +8077,7 @@
         <v/>
       </c>
       <c r="K130" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>F3 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="131">
@@ -8024,10 +8085,10 @@
         <v>128</v>
       </c>
       <c r="B131" t="str">
-        <v>HM010</v>
+        <v>HM025</v>
       </c>
       <c r="C131" t="str">
-        <v>Bridge of Voices</v>
+        <v>Deep Digs</v>
       </c>
       <c r="D131" t="str">
         <v>Hybrid</v>
@@ -8036,22 +8097,22 @@
         <v>Team Leader</v>
       </c>
       <c r="F131" t="str">
-        <v>Hetvi Patel</v>
+        <v>RUDRA JOSHI</v>
       </c>
       <c r="G131" t="str">
-        <v>240410111007</v>
+        <v>24041011039</v>
       </c>
       <c r="H131" t="str">
-        <v>6359349090</v>
+        <v>8866052251</v>
       </c>
       <c r="I131" t="str">
-        <v>24ec28@svitvasad.ac.in</v>
+        <v>rudraashu4@gmail.com</v>
       </c>
       <c r="J131" t="str">
-        <v>Electronics &amp; Communication (EC)</v>
+        <v>Information Technology (IT)</v>
       </c>
       <c r="K131" t="str">
-        <v>F6 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="132">
@@ -8059,10 +8120,10 @@
         <v>129</v>
       </c>
       <c r="B132" t="str">
-        <v>HM010</v>
+        <v>HM025</v>
       </c>
       <c r="C132" t="str">
-        <v>Bridge of Voices</v>
+        <v>Deep Digs</v>
       </c>
       <c r="D132" t="str">
         <v>Hybrid</v>
@@ -8071,13 +8132,13 @@
         <v>Member 1</v>
       </c>
       <c r="F132" t="str">
-        <v>Anjali Jayswal</v>
+        <v>Aditya Shah</v>
       </c>
       <c r="G132" t="str">
-        <v>240410111004</v>
+        <v>240410116001</v>
       </c>
       <c r="H132" t="str">
-        <v>9574541530</v>
+        <v>8849100417</v>
       </c>
       <c r="I132" t="str">
         <v/>
@@ -8086,7 +8147,7 @@
         <v/>
       </c>
       <c r="K132" t="str">
-        <v>F6 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="133">
@@ -8094,10 +8155,10 @@
         <v>130</v>
       </c>
       <c r="B133" t="str">
-        <v>HM010</v>
+        <v>HM025</v>
       </c>
       <c r="C133" t="str">
-        <v>Bridge of Voices</v>
+        <v>Deep Digs</v>
       </c>
       <c r="D133" t="str">
         <v>Hybrid</v>
@@ -8106,13 +8167,13 @@
         <v>Member 2</v>
       </c>
       <c r="F133" t="str">
-        <v>Gopi Patel</v>
+        <v>Deep Padhiyar</v>
       </c>
       <c r="G133" t="str">
-        <v>240410111017</v>
+        <v>240410116017</v>
       </c>
       <c r="H133" t="str">
-        <v>9328894722</v>
+        <v>9016622658</v>
       </c>
       <c r="I133" t="str">
         <v/>
@@ -8121,7 +8182,7 @@
         <v/>
       </c>
       <c r="K133" t="str">
-        <v>F6 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="134">
@@ -8129,10 +8190,10 @@
         <v>131</v>
       </c>
       <c r="B134" t="str">
-        <v>HM010</v>
+        <v>HM025</v>
       </c>
       <c r="C134" t="str">
-        <v>Bridge of Voices</v>
+        <v>Deep Digs</v>
       </c>
       <c r="D134" t="str">
         <v>Hybrid</v>
@@ -8141,13 +8202,13 @@
         <v>Member 3</v>
       </c>
       <c r="F134" t="str">
-        <v>Bansi Patel</v>
+        <v>Meet Makvana</v>
       </c>
       <c r="G134" t="str">
-        <v>240410116069</v>
+        <v>240410116045</v>
       </c>
       <c r="H134" t="str">
-        <v>7990435587</v>
+        <v>7016808631</v>
       </c>
       <c r="I134" t="str">
         <v/>
@@ -8156,7 +8217,7 @@
         <v/>
       </c>
       <c r="K134" t="str">
-        <v>F6 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="135">
@@ -8164,10 +8225,10 @@
         <v>132</v>
       </c>
       <c r="B135" t="str">
-        <v>HM004</v>
+        <v>HM010</v>
       </c>
       <c r="C135" t="str">
-        <v>VoltVision</v>
+        <v>Bridge of Voices</v>
       </c>
       <c r="D135" t="str">
         <v>Hybrid</v>
@@ -8176,22 +8237,22 @@
         <v>Team Leader</v>
       </c>
       <c r="F135" t="str">
-        <v>Lakshyaa gaurang shah</v>
+        <v>Hetvi Patel</v>
       </c>
       <c r="G135" t="str">
-        <v>240410111025</v>
+        <v>240410111007</v>
       </c>
       <c r="H135" t="str">
-        <v>8320867346</v>
+        <v>6359349090</v>
       </c>
       <c r="I135" t="str">
-        <v>shahlakshyaa901@gmail.com</v>
+        <v>24ec28@svitvasad.ac.in</v>
       </c>
       <c r="J135" t="str">
         <v>Electronics &amp; Communication (EC)</v>
       </c>
       <c r="K135" t="str">
-        <v>S3 Lab Second floor CE dept.</v>
+        <v>F6 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="136">
@@ -8199,10 +8260,10 @@
         <v>133</v>
       </c>
       <c r="B136" t="str">
-        <v>HM004</v>
+        <v>HM010</v>
       </c>
       <c r="C136" t="str">
-        <v>VoltVision</v>
+        <v>Bridge of Voices</v>
       </c>
       <c r="D136" t="str">
         <v>Hybrid</v>
@@ -8211,13 +8272,13 @@
         <v>Member 1</v>
       </c>
       <c r="F136" t="str">
-        <v>Taksha Adhyaru</v>
+        <v>Anjali Jayswal</v>
       </c>
       <c r="G136" t="str">
-        <v>240410111003</v>
+        <v>240410111004</v>
       </c>
       <c r="H136" t="str">
-        <v>9409233040</v>
+        <v>9574541530</v>
       </c>
       <c r="I136" t="str">
         <v/>
@@ -8226,7 +8287,7 @@
         <v/>
       </c>
       <c r="K136" t="str">
-        <v>S3 Lab Second floor CE dept.</v>
+        <v>F6 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="137">
@@ -8234,10 +8295,10 @@
         <v>134</v>
       </c>
       <c r="B137" t="str">
-        <v>HM004</v>
+        <v>HM010</v>
       </c>
       <c r="C137" t="str">
-        <v>VoltVision</v>
+        <v>Bridge of Voices</v>
       </c>
       <c r="D137" t="str">
         <v>Hybrid</v>
@@ -8246,13 +8307,13 @@
         <v>Member 2</v>
       </c>
       <c r="F137" t="str">
-        <v>Aatman joshi</v>
+        <v>Gopi Patel</v>
       </c>
       <c r="G137" t="str">
-        <v>240410111002</v>
+        <v>240410111017</v>
       </c>
       <c r="H137" t="str">
-        <v>9104118105</v>
+        <v>9328894722</v>
       </c>
       <c r="I137" t="str">
         <v/>
@@ -8261,7 +8322,7 @@
         <v/>
       </c>
       <c r="K137" t="str">
-        <v>S3 Lab Second floor CE dept.</v>
+        <v>F6 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="138">
@@ -8269,10 +8330,10 @@
         <v>135</v>
       </c>
       <c r="B138" t="str">
-        <v>HM004</v>
+        <v>HM010</v>
       </c>
       <c r="C138" t="str">
-        <v>VoltVision</v>
+        <v>Bridge of Voices</v>
       </c>
       <c r="D138" t="str">
         <v>Hybrid</v>
@@ -8281,13 +8342,13 @@
         <v>Member 3</v>
       </c>
       <c r="F138" t="str">
-        <v>vinay nambiar</v>
+        <v>Bansi Patel</v>
       </c>
       <c r="G138" t="str">
-        <v>240410111012</v>
+        <v>240410116069</v>
       </c>
       <c r="H138" t="str">
-        <v>7436043304</v>
+        <v>7990435587</v>
       </c>
       <c r="I138" t="str">
         <v/>
@@ -8296,7 +8357,7 @@
         <v/>
       </c>
       <c r="K138" t="str">
-        <v>S3 Lab Second floor CE dept.</v>
+        <v>F6 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="139">
@@ -8304,10 +8365,10 @@
         <v>136</v>
       </c>
       <c r="B139" t="str">
-        <v>HM012</v>
+        <v>HM004</v>
       </c>
       <c r="C139" t="str">
-        <v>Mech Innovators</v>
+        <v>VoltVision</v>
       </c>
       <c r="D139" t="str">
         <v>Hybrid</v>
@@ -8316,22 +8377,22 @@
         <v>Team Leader</v>
       </c>
       <c r="F139" t="str">
-        <v>Swayam Shah</v>
+        <v>Lakshyaa gaurang shah</v>
       </c>
       <c r="G139" t="str">
-        <v>240410119045</v>
+        <v>240410111025</v>
       </c>
       <c r="H139" t="str">
-        <v>9265294869</v>
+        <v>8320867346</v>
       </c>
       <c r="I139" t="str">
-        <v>24m25@svitvasad.ac.in</v>
+        <v>shahlakshyaa901@gmail.com</v>
       </c>
       <c r="J139" t="str">
-        <v>Mechanical Engineering (ME)</v>
+        <v>Electronics &amp; Communication (EC)</v>
       </c>
       <c r="K139" t="str">
-        <v>F1 Lab First floor CE dept.</v>
+        <v>S3 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="140">
@@ -8339,10 +8400,10 @@
         <v>137</v>
       </c>
       <c r="B140" t="str">
-        <v>HM012</v>
+        <v>HM004</v>
       </c>
       <c r="C140" t="str">
-        <v>Mech Innovators</v>
+        <v>VoltVision</v>
       </c>
       <c r="D140" t="str">
         <v>Hybrid</v>
@@ -8351,13 +8412,13 @@
         <v>Member 1</v>
       </c>
       <c r="F140" t="str">
-        <v>Dharmik Sanathara</v>
+        <v>Taksha Adhyaru</v>
       </c>
       <c r="G140" t="str">
-        <v>240410119043</v>
+        <v>240410111003</v>
       </c>
       <c r="H140" t="str">
-        <v>7046071284</v>
+        <v>9409233040</v>
       </c>
       <c r="I140" t="str">
         <v/>
@@ -8366,7 +8427,7 @@
         <v/>
       </c>
       <c r="K140" t="str">
-        <v>F1 Lab First floor CE dept.</v>
+        <v>S3 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="141">
@@ -8374,10 +8435,10 @@
         <v>138</v>
       </c>
       <c r="B141" t="str">
-        <v>HM012</v>
+        <v>HM004</v>
       </c>
       <c r="C141" t="str">
-        <v>Mech Innovators</v>
+        <v>VoltVision</v>
       </c>
       <c r="D141" t="str">
         <v>Hybrid</v>
@@ -8386,13 +8447,13 @@
         <v>Member 2</v>
       </c>
       <c r="F141" t="str">
-        <v>Milan Vanzara</v>
+        <v>Aatman joshi</v>
       </c>
       <c r="G141" t="str">
-        <v>240410119050</v>
+        <v>240410111002</v>
       </c>
       <c r="H141" t="str">
-        <v>9909549543</v>
+        <v>9104118105</v>
       </c>
       <c r="I141" t="str">
         <v/>
@@ -8401,7 +8462,7 @@
         <v/>
       </c>
       <c r="K141" t="str">
-        <v>F1 Lab First floor CE dept.</v>
+        <v>S3 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="142">
@@ -8409,10 +8470,10 @@
         <v>139</v>
       </c>
       <c r="B142" t="str">
-        <v>HM012</v>
+        <v>HM004</v>
       </c>
       <c r="C142" t="str">
-        <v>Mech Innovators</v>
+        <v>VoltVision</v>
       </c>
       <c r="D142" t="str">
         <v>Hybrid</v>
@@ -8421,13 +8482,13 @@
         <v>Member 3</v>
       </c>
       <c r="F142" t="str">
-        <v>Pursharth Singh</v>
+        <v>vinay nambiar</v>
       </c>
       <c r="G142" t="str">
-        <v>240410119039</v>
+        <v>240410111012</v>
       </c>
       <c r="H142" t="str">
-        <v>8490835681</v>
+        <v>7436043304</v>
       </c>
       <c r="I142" t="str">
         <v/>
@@ -8436,7 +8497,7 @@
         <v/>
       </c>
       <c r="K142" t="str">
-        <v>F1 Lab First floor CE dept.</v>
+        <v>S3 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="143">
@@ -8444,10 +8505,10 @@
         <v>140</v>
       </c>
       <c r="B143" t="str">
-        <v>HM013</v>
+        <v>HM012</v>
       </c>
       <c r="C143" t="str">
-        <v>Agrisense</v>
+        <v>Mech Innovators</v>
       </c>
       <c r="D143" t="str">
         <v>Hybrid</v>
@@ -8456,22 +8517,22 @@
         <v>Team Leader</v>
       </c>
       <c r="F143" t="str">
-        <v>CHAITANYA GIRI</v>
+        <v>Swayam Shah</v>
       </c>
       <c r="G143" t="str">
-        <v>230410149016</v>
+        <v>240410119045</v>
       </c>
       <c r="H143" t="str">
-        <v>9327942604</v>
+        <v>9265294869</v>
       </c>
       <c r="I143" t="str">
-        <v>23csd62@svitvasad.ac.in</v>
+        <v>24m25@svitvasad.ac.in</v>
       </c>
       <c r="J143" t="str">
-        <v>Computer Science &amp; Design (CSD)</v>
+        <v>Mechanical Engineering (ME)</v>
       </c>
       <c r="K143" t="str">
-        <v>G3 Lab Ground floor CE dept.</v>
+        <v>F1 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="144">
@@ -8479,10 +8540,10 @@
         <v>141</v>
       </c>
       <c r="B144" t="str">
-        <v>HM013</v>
+        <v>HM012</v>
       </c>
       <c r="C144" t="str">
-        <v>Agrisense</v>
+        <v>Mech Innovators</v>
       </c>
       <c r="D144" t="str">
         <v>Hybrid</v>
@@ -8491,13 +8552,13 @@
         <v>Member 1</v>
       </c>
       <c r="F144" t="str">
-        <v>Aarsh Patel</v>
+        <v>Dharmik Sanathara</v>
       </c>
       <c r="G144" t="str">
-        <v>230410149001</v>
+        <v>240410119043</v>
       </c>
       <c r="H144" t="str">
-        <v>7984277728</v>
+        <v>7046071284</v>
       </c>
       <c r="I144" t="str">
         <v/>
@@ -8506,7 +8567,7 @@
         <v/>
       </c>
       <c r="K144" t="str">
-        <v>G3 Lab Ground floor CE dept.</v>
+        <v>F1 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="145">
@@ -8514,10 +8575,10 @@
         <v>142</v>
       </c>
       <c r="B145" t="str">
-        <v>HM013</v>
+        <v>HM012</v>
       </c>
       <c r="C145" t="str">
-        <v>Agrisense</v>
+        <v>Mech Innovators</v>
       </c>
       <c r="D145" t="str">
         <v>Hybrid</v>
@@ -8526,13 +8587,13 @@
         <v>Member 2</v>
       </c>
       <c r="F145" t="str">
-        <v>Hetanshi Suthar</v>
+        <v>Milan Vanzara</v>
       </c>
       <c r="G145" t="str">
-        <v>230410107131</v>
+        <v>240410119050</v>
       </c>
       <c r="H145" t="str">
-        <v>9824077988</v>
+        <v>9909549543</v>
       </c>
       <c r="I145" t="str">
         <v/>
@@ -8541,7 +8602,7 @@
         <v/>
       </c>
       <c r="K145" t="str">
-        <v>G3 Lab Ground floor CE dept.</v>
+        <v>F1 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="146">
@@ -8549,10 +8610,10 @@
         <v>143</v>
       </c>
       <c r="B146" t="str">
-        <v>HM013</v>
+        <v>HM012</v>
       </c>
       <c r="C146" t="str">
-        <v>Agrisense</v>
+        <v>Mech Innovators</v>
       </c>
       <c r="D146" t="str">
         <v>Hybrid</v>
@@ -8561,13 +8622,13 @@
         <v>Member 3</v>
       </c>
       <c r="F146" t="str">
-        <v>Parth Bhatti</v>
+        <v>Pursharth Singh</v>
       </c>
       <c r="G146" t="str">
-        <v>240413107001</v>
+        <v>240410119039</v>
       </c>
       <c r="H146" t="str">
-        <v>8160695465</v>
+        <v>8490835681</v>
       </c>
       <c r="I146" t="str">
         <v/>
@@ -8576,7 +8637,7 @@
         <v/>
       </c>
       <c r="K146" t="str">
-        <v>G3 Lab Ground floor CE dept.</v>
+        <v>F1 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="147">
@@ -8584,10 +8645,10 @@
         <v>144</v>
       </c>
       <c r="B147" t="str">
-        <v>HM008</v>
+        <v>HM013</v>
       </c>
       <c r="C147" t="str">
-        <v>Waveminds</v>
+        <v>Agrisense</v>
       </c>
       <c r="D147" t="str">
         <v>Hybrid</v>
@@ -8596,22 +8657,22 @@
         <v>Team Leader</v>
       </c>
       <c r="F147" t="str">
-        <v>Aryan Shah</v>
+        <v>CHAITANYA GIRI</v>
       </c>
       <c r="G147" t="str">
-        <v>240410111023</v>
+        <v>230410149016</v>
       </c>
       <c r="H147" t="str">
-        <v>9104513714</v>
+        <v>9327942604</v>
       </c>
       <c r="I147" t="str">
-        <v>shaharyan1726@gmail.com</v>
+        <v>23csd62@svitvasad.ac.in</v>
       </c>
       <c r="J147" t="str">
-        <v>Electronics &amp; Communication (EC)</v>
+        <v>Computer Science &amp; Design (CSD)</v>
       </c>
       <c r="K147" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>G3 Lab Ground floor CE dept.</v>
       </c>
     </row>
     <row r="148">
@@ -8619,10 +8680,10 @@
         <v>145</v>
       </c>
       <c r="B148" t="str">
-        <v>HM008</v>
+        <v>HM013</v>
       </c>
       <c r="C148" t="str">
-        <v>Waveminds</v>
+        <v>Agrisense</v>
       </c>
       <c r="D148" t="str">
         <v>Hybrid</v>
@@ -8631,13 +8692,13 @@
         <v>Member 1</v>
       </c>
       <c r="F148" t="str">
-        <v>Aarav Shah</v>
+        <v>Aarsh Patel</v>
       </c>
       <c r="G148" t="str">
-        <v>240410111022</v>
+        <v>230410149001</v>
       </c>
       <c r="H148" t="str">
-        <v>6352283738</v>
+        <v>7984277728</v>
       </c>
       <c r="I148" t="str">
         <v/>
@@ -8646,7 +8707,7 @@
         <v/>
       </c>
       <c r="K148" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>G3 Lab Ground floor CE dept.</v>
       </c>
     </row>
     <row r="149">
@@ -8654,10 +8715,10 @@
         <v>146</v>
       </c>
       <c r="B149" t="str">
-        <v>HM008</v>
+        <v>HM013</v>
       </c>
       <c r="C149" t="str">
-        <v>Waveminds</v>
+        <v>Agrisense</v>
       </c>
       <c r="D149" t="str">
         <v>Hybrid</v>
@@ -8666,13 +8727,13 @@
         <v>Member 2</v>
       </c>
       <c r="F149" t="str">
-        <v>Santanu Khanra</v>
+        <v>Hetanshi Suthar</v>
       </c>
       <c r="G149" t="str">
-        <v>240410111008</v>
+        <v>230410107131</v>
       </c>
       <c r="H149" t="str">
-        <v>8347400659</v>
+        <v>9824077988</v>
       </c>
       <c r="I149" t="str">
         <v/>
@@ -8681,7 +8742,7 @@
         <v/>
       </c>
       <c r="K149" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>G3 Lab Ground floor CE dept.</v>
       </c>
     </row>
     <row r="150">
@@ -8689,10 +8750,10 @@
         <v>147</v>
       </c>
       <c r="B150" t="str">
-        <v>HM008</v>
+        <v>HM013</v>
       </c>
       <c r="C150" t="str">
-        <v>Waveminds</v>
+        <v>Agrisense</v>
       </c>
       <c r="D150" t="str">
         <v>Hybrid</v>
@@ -8701,13 +8762,13 @@
         <v>Member 3</v>
       </c>
       <c r="F150" t="str">
-        <v>Parv Baxi</v>
+        <v>Parth Bhatti</v>
       </c>
       <c r="G150" t="str">
-        <v>2504131110010</v>
+        <v>240413107001</v>
       </c>
       <c r="H150" t="str">
-        <v>9313322432</v>
+        <v>8160695465</v>
       </c>
       <c r="I150" t="str">
         <v/>
@@ -8716,7 +8777,7 @@
         <v/>
       </c>
       <c r="K150" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>G3 Lab Ground floor CE dept.</v>
       </c>
     </row>
     <row r="151">
@@ -8724,10 +8785,10 @@
         <v>148</v>
       </c>
       <c r="B151" t="str">
-        <v>HM006</v>
+        <v>HM008</v>
       </c>
       <c r="C151" t="str">
-        <v>AeroMorph</v>
+        <v>Waveminds</v>
       </c>
       <c r="D151" t="str">
         <v>Hybrid</v>
@@ -8736,19 +8797,19 @@
         <v>Team Leader</v>
       </c>
       <c r="F151" t="str">
-        <v>Jadav Anvi</v>
+        <v>Aryan Shah</v>
       </c>
       <c r="G151" t="str">
-        <v>230410101012</v>
+        <v>240410111023</v>
       </c>
       <c r="H151" t="str">
-        <v>7984801132</v>
+        <v>9104513714</v>
       </c>
       <c r="I151" t="str">
-        <v>jadavanvi2006@gmail.com</v>
+        <v>shaharyan1726@gmail.com</v>
       </c>
       <c r="J151" t="str">
-        <v>Aeronautical Engineering</v>
+        <v>Electronics &amp; Communication (EC)</v>
       </c>
       <c r="K151" t="str">
         <v>F5 Lab First floor CE dept.</v>
@@ -8759,10 +8820,10 @@
         <v>149</v>
       </c>
       <c r="B152" t="str">
-        <v>HM006</v>
+        <v>HM008</v>
       </c>
       <c r="C152" t="str">
-        <v>AeroMorph</v>
+        <v>Waveminds</v>
       </c>
       <c r="D152" t="str">
         <v>Hybrid</v>
@@ -8771,13 +8832,13 @@
         <v>Member 1</v>
       </c>
       <c r="F152" t="str">
-        <v>Tisha Pandya</v>
+        <v>Aarav Shah</v>
       </c>
       <c r="G152" t="str">
-        <v>230410101012</v>
+        <v>240410111022</v>
       </c>
       <c r="H152" t="str">
-        <v>9327552539</v>
+        <v>6352283738</v>
       </c>
       <c r="I152" t="str">
         <v/>
@@ -8794,10 +8855,10 @@
         <v>150</v>
       </c>
       <c r="B153" t="str">
-        <v>HM006</v>
+        <v>HM008</v>
       </c>
       <c r="C153" t="str">
-        <v>AeroMorph</v>
+        <v>Waveminds</v>
       </c>
       <c r="D153" t="str">
         <v>Hybrid</v>
@@ -8806,13 +8867,13 @@
         <v>Member 2</v>
       </c>
       <c r="F153" t="str">
-        <v>Raj Bhanushali</v>
+        <v>Santanu Khanra</v>
       </c>
       <c r="G153" t="str">
-        <v>240410119041</v>
+        <v>240410111008</v>
       </c>
       <c r="H153" t="str">
-        <v>6352926621</v>
+        <v>8347400659</v>
       </c>
       <c r="I153" t="str">
         <v/>
@@ -8829,10 +8890,10 @@
         <v>151</v>
       </c>
       <c r="B154" t="str">
-        <v>HM006</v>
+        <v>HM008</v>
       </c>
       <c r="C154" t="str">
-        <v>AeroMorph</v>
+        <v>Waveminds</v>
       </c>
       <c r="D154" t="str">
         <v>Hybrid</v>
@@ -8841,13 +8902,13 @@
         <v>Member 3</v>
       </c>
       <c r="F154" t="str">
-        <v>Ajaya Mishra</v>
+        <v>Parv Baxi</v>
       </c>
       <c r="G154" t="str">
-        <v>230410101024</v>
+        <v>2504131110010</v>
       </c>
       <c r="H154" t="str">
-        <v>9979954999</v>
+        <v>9313322432</v>
       </c>
       <c r="I154" t="str">
         <v/>
@@ -8864,10 +8925,10 @@
         <v>152</v>
       </c>
       <c r="B155" t="str">
-        <v>HM009</v>
+        <v>HM006</v>
       </c>
       <c r="C155" t="str">
-        <v>AgriMix Pro</v>
+        <v>AeroMorph</v>
       </c>
       <c r="D155" t="str">
         <v>Hybrid</v>
@@ -8876,22 +8937,22 @@
         <v>Team Leader</v>
       </c>
       <c r="F155" t="str">
-        <v>prajapati pratham</v>
+        <v>Jadav Anvi</v>
       </c>
       <c r="G155" t="str">
-        <v>250410111022</v>
+        <v>230410101012</v>
       </c>
       <c r="H155" t="str">
-        <v>9409766800</v>
+        <v>7984801132</v>
       </c>
       <c r="I155" t="str">
-        <v>prajapati12345pratham@gmail.com</v>
+        <v>jadavanvi2006@gmail.com</v>
       </c>
       <c r="J155" t="str">
-        <v>Electronics &amp; Communication (EC)</v>
+        <v>Aeronautical Engineering</v>
       </c>
       <c r="K155" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="156">
@@ -8899,10 +8960,10 @@
         <v>153</v>
       </c>
       <c r="B156" t="str">
-        <v>HM009</v>
+        <v>HM006</v>
       </c>
       <c r="C156" t="str">
-        <v>AgriMix Pro</v>
+        <v>AeroMorph</v>
       </c>
       <c r="D156" t="str">
         <v>Hybrid</v>
@@ -8911,13 +8972,13 @@
         <v>Member 1</v>
       </c>
       <c r="F156" t="str">
-        <v>Savya singh</v>
+        <v>Tisha Pandya</v>
       </c>
       <c r="G156" t="str">
-        <v>250410116119</v>
+        <v>230410101012</v>
       </c>
       <c r="H156" t="str">
-        <v>9974322090</v>
+        <v>9327552539</v>
       </c>
       <c r="I156" t="str">
         <v/>
@@ -8926,7 +8987,7 @@
         <v/>
       </c>
       <c r="K156" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="157">
@@ -8934,10 +8995,10 @@
         <v>154</v>
       </c>
       <c r="B157" t="str">
-        <v>HM009</v>
+        <v>HM006</v>
       </c>
       <c r="C157" t="str">
-        <v>AgriMix Pro</v>
+        <v>AeroMorph</v>
       </c>
       <c r="D157" t="str">
         <v>Hybrid</v>
@@ -8946,13 +9007,13 @@
         <v>Member 2</v>
       </c>
       <c r="F157" t="str">
-        <v>Drasti bodana</v>
+        <v>Raj Bhanushali</v>
       </c>
       <c r="G157" t="str">
-        <v>250410116009</v>
+        <v>240410119041</v>
       </c>
       <c r="H157" t="str">
-        <v>9313323735</v>
+        <v>6352926621</v>
       </c>
       <c r="I157" t="str">
         <v/>
@@ -8961,7 +9022,7 @@
         <v/>
       </c>
       <c r="K157" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="158">
@@ -8969,10 +9030,10 @@
         <v>155</v>
       </c>
       <c r="B158" t="str">
-        <v>HM009</v>
+        <v>HM006</v>
       </c>
       <c r="C158" t="str">
-        <v>AgriMix Pro</v>
+        <v>AeroMorph</v>
       </c>
       <c r="D158" t="str">
         <v>Hybrid</v>
@@ -8981,13 +9042,13 @@
         <v>Member 3</v>
       </c>
       <c r="F158" t="str">
-        <v>Bhavya sharma</v>
+        <v>Ajaya Mishra</v>
       </c>
       <c r="G158" t="str">
-        <v>250410116114</v>
+        <v>230410101024</v>
       </c>
       <c r="H158" t="str">
-        <v>9106650125</v>
+        <v>9979954999</v>
       </c>
       <c r="I158" t="str">
         <v/>
@@ -8996,7 +9057,7 @@
         <v/>
       </c>
       <c r="K158" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="159">
@@ -9004,10 +9065,10 @@
         <v>156</v>
       </c>
       <c r="B159" t="str">
-        <v>HM005</v>
+        <v>HM009</v>
       </c>
       <c r="C159" t="str">
-        <v>FusionSpark</v>
+        <v>AgriMix Pro</v>
       </c>
       <c r="D159" t="str">
         <v>Hybrid</v>
@@ -9016,22 +9077,22 @@
         <v>Team Leader</v>
       </c>
       <c r="F159" t="str">
-        <v>ISHA SHAH</v>
+        <v>prajapati pratham</v>
       </c>
       <c r="G159" t="str">
-        <v>240410111024</v>
+        <v>250410111022</v>
       </c>
       <c r="H159" t="str">
-        <v>9426661449</v>
+        <v>9409766800</v>
       </c>
       <c r="I159" t="str">
-        <v>ishashah2656@gmail.com</v>
+        <v>prajapati12345pratham@gmail.com</v>
       </c>
       <c r="J159" t="str">
         <v>Electronics &amp; Communication (EC)</v>
       </c>
       <c r="K159" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="160">
@@ -9039,10 +9100,10 @@
         <v>157</v>
       </c>
       <c r="B160" t="str">
-        <v>HM005</v>
+        <v>HM009</v>
       </c>
       <c r="C160" t="str">
-        <v>FusionSpark</v>
+        <v>AgriMix Pro</v>
       </c>
       <c r="D160" t="str">
         <v>Hybrid</v>
@@ -9051,13 +9112,13 @@
         <v>Member 1</v>
       </c>
       <c r="F160" t="str">
-        <v>KAVYA DAVE</v>
+        <v>Savya singh</v>
       </c>
       <c r="G160" t="str">
-        <v>240410116110</v>
+        <v>250410116119</v>
       </c>
       <c r="H160" t="str">
-        <v>8866201745</v>
+        <v>9974322090</v>
       </c>
       <c r="I160" t="str">
         <v/>
@@ -9066,7 +9127,7 @@
         <v/>
       </c>
       <c r="K160" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="161">
@@ -9074,10 +9135,10 @@
         <v>158</v>
       </c>
       <c r="B161" t="str">
-        <v>HM005</v>
+        <v>HM009</v>
       </c>
       <c r="C161" t="str">
-        <v>FusionSpark</v>
+        <v>AgriMix Pro</v>
       </c>
       <c r="D161" t="str">
         <v>Hybrid</v>
@@ -9086,13 +9147,13 @@
         <v>Member 2</v>
       </c>
       <c r="F161" t="str">
-        <v>ADITYA VALAND</v>
+        <v>Drasti bodana</v>
       </c>
       <c r="G161" t="str">
-        <v>240410116136</v>
+        <v>250410116009</v>
       </c>
       <c r="H161" t="str">
-        <v>8488880596</v>
+        <v>9313323735</v>
       </c>
       <c r="I161" t="str">
         <v/>
@@ -9101,7 +9162,7 @@
         <v/>
       </c>
       <c r="K161" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="162">
@@ -9109,10 +9170,10 @@
         <v>159</v>
       </c>
       <c r="B162" t="str">
-        <v>HM005</v>
+        <v>HM009</v>
       </c>
       <c r="C162" t="str">
-        <v>FusionSpark</v>
+        <v>AgriMix Pro</v>
       </c>
       <c r="D162" t="str">
         <v>Hybrid</v>
@@ -9121,13 +9182,13 @@
         <v>Member 3</v>
       </c>
       <c r="F162" t="str">
-        <v>JENIL SHINGALA</v>
+        <v>Bhavya sharma</v>
       </c>
       <c r="G162" t="str">
-        <v>240410116120</v>
+        <v>250410116114</v>
       </c>
       <c r="H162" t="str">
-        <v>8799230510</v>
+        <v>9106650125</v>
       </c>
       <c r="I162" t="str">
         <v/>
@@ -9136,7 +9197,7 @@
         <v/>
       </c>
       <c r="K162" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="163">
@@ -9144,10 +9205,10 @@
         <v>160</v>
       </c>
       <c r="B163" t="str">
-        <v>HM019</v>
+        <v>HM005</v>
       </c>
       <c r="C163" t="str">
-        <v>Fifty Shades Of Cache</v>
+        <v>FusionSpark</v>
       </c>
       <c r="D163" t="str">
         <v>Hybrid</v>
@@ -9156,22 +9217,22 @@
         <v>Team Leader</v>
       </c>
       <c r="F163" t="str">
-        <v>Agneloze Williams</v>
+        <v>ISHA SHAH</v>
       </c>
       <c r="G163" t="str">
-        <v>250410107204</v>
+        <v>240410111024</v>
       </c>
       <c r="H163" t="str">
-        <v>9638241325</v>
+        <v>9426661449</v>
       </c>
       <c r="I163" t="str">
-        <v>agnelozesw@gmail.com</v>
+        <v>ishashah2656@gmail.com</v>
       </c>
       <c r="J163" t="str">
-        <v>Computer Engineering (CE)</v>
+        <v>Electronics &amp; Communication (EC)</v>
       </c>
       <c r="K163" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="164">
@@ -9179,10 +9240,10 @@
         <v>161</v>
       </c>
       <c r="B164" t="str">
-        <v>HM019</v>
+        <v>HM005</v>
       </c>
       <c r="C164" t="str">
-        <v>Fifty Shades Of Cache</v>
+        <v>FusionSpark</v>
       </c>
       <c r="D164" t="str">
         <v>Hybrid</v>
@@ -9191,13 +9252,13 @@
         <v>Member 1</v>
       </c>
       <c r="F164" t="str">
-        <v>Zinkal Gadiya</v>
+        <v>KAVYA DAVE</v>
       </c>
       <c r="G164" t="str">
-        <v>250410107036</v>
+        <v>240410116110</v>
       </c>
       <c r="H164" t="str">
-        <v>9726564632</v>
+        <v>8866201745</v>
       </c>
       <c r="I164" t="str">
         <v/>
@@ -9206,7 +9267,7 @@
         <v/>
       </c>
       <c r="K164" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="165">
@@ -9214,10 +9275,10 @@
         <v>162</v>
       </c>
       <c r="B165" t="str">
-        <v>HM019</v>
+        <v>HM005</v>
       </c>
       <c r="C165" t="str">
-        <v>Fifty Shades Of Cache</v>
+        <v>FusionSpark</v>
       </c>
       <c r="D165" t="str">
         <v>Hybrid</v>
@@ -9226,13 +9287,13 @@
         <v>Member 2</v>
       </c>
       <c r="F165" t="str">
-        <v>Deep Thakkar</v>
+        <v>ADITYA VALAND</v>
       </c>
       <c r="G165" t="str">
-        <v>250410107190</v>
+        <v>240410116136</v>
       </c>
       <c r="H165" t="str">
-        <v>9428982851</v>
+        <v>8488880596</v>
       </c>
       <c r="I165" t="str">
         <v/>
@@ -9241,7 +9302,7 @@
         <v/>
       </c>
       <c r="K165" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="166">
@@ -9249,10 +9310,10 @@
         <v>163</v>
       </c>
       <c r="B166" t="str">
-        <v>HM019</v>
+        <v>HM005</v>
       </c>
       <c r="C166" t="str">
-        <v>Fifty Shades Of Cache</v>
+        <v>FusionSpark</v>
       </c>
       <c r="D166" t="str">
         <v>Hybrid</v>
@@ -9261,13 +9322,13 @@
         <v>Member 3</v>
       </c>
       <c r="F166" t="str">
-        <v>Neev Patel</v>
+        <v>JENIL SHINGALA</v>
       </c>
       <c r="G166" t="str">
-        <v>250410107122</v>
+        <v>240410116120</v>
       </c>
       <c r="H166" t="str">
-        <v>9429400440</v>
+        <v>8799230510</v>
       </c>
       <c r="I166" t="str">
         <v/>
@@ -9276,7 +9337,7 @@
         <v/>
       </c>
       <c r="K166" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="167">
@@ -9284,10 +9345,10 @@
         <v>164</v>
       </c>
       <c r="B167" t="str">
-        <v>HM017</v>
+        <v>HM019</v>
       </c>
       <c r="C167" t="str">
-        <v>Sky sketchers</v>
+        <v>Fifty Shades Of Cache</v>
       </c>
       <c r="D167" t="str">
         <v>Hybrid</v>
@@ -9296,22 +9357,22 @@
         <v>Team Leader</v>
       </c>
       <c r="F167" t="str">
-        <v>Patel Aum Dhiren</v>
+        <v>Agneloze Williams</v>
       </c>
       <c r="G167" t="str">
-        <v>250413101009</v>
+        <v>250410107204</v>
       </c>
       <c r="H167" t="str">
-        <v>8320950668</v>
+        <v>9638241325</v>
       </c>
       <c r="I167" t="str">
-        <v>patelaum2266@gmail.com</v>
+        <v>agnelozesw@gmail.com</v>
       </c>
       <c r="J167" t="str">
-        <v>Aeronautical Engineering</v>
+        <v>Computer Engineering (CE)</v>
       </c>
       <c r="K167" t="str">
-        <v>F1 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="168">
@@ -9319,10 +9380,10 @@
         <v>165</v>
       </c>
       <c r="B168" t="str">
-        <v>HM017</v>
+        <v>HM019</v>
       </c>
       <c r="C168" t="str">
-        <v>Sky sketchers</v>
+        <v>Fifty Shades Of Cache</v>
       </c>
       <c r="D168" t="str">
         <v>Hybrid</v>
@@ -9331,13 +9392,13 @@
         <v>Member 1</v>
       </c>
       <c r="F168" t="str">
-        <v>Patel Ayush Saurabh</v>
+        <v>Zinkal Gadiya</v>
       </c>
       <c r="G168" t="str">
-        <v>250413101010</v>
+        <v>250410107036</v>
       </c>
       <c r="H168" t="str">
-        <v>9023800699</v>
+        <v>9726564632</v>
       </c>
       <c r="I168" t="str">
         <v/>
@@ -9346,7 +9407,7 @@
         <v/>
       </c>
       <c r="K168" t="str">
-        <v>F1 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="169">
@@ -9354,10 +9415,10 @@
         <v>166</v>
       </c>
       <c r="B169" t="str">
-        <v>HM017</v>
+        <v>HM019</v>
       </c>
       <c r="C169" t="str">
-        <v>Sky sketchers</v>
+        <v>Fifty Shades Of Cache</v>
       </c>
       <c r="D169" t="str">
         <v>Hybrid</v>
@@ -9366,13 +9427,13 @@
         <v>Member 2</v>
       </c>
       <c r="F169" t="str">
-        <v>Patel Devesh Yogesh</v>
+        <v>Deep Thakkar</v>
       </c>
       <c r="G169" t="str">
-        <v>250413101002</v>
+        <v>250410107190</v>
       </c>
       <c r="H169" t="str">
-        <v>8160771388</v>
+        <v>9428982851</v>
       </c>
       <c r="I169" t="str">
         <v/>
@@ -9381,7 +9442,7 @@
         <v/>
       </c>
       <c r="K169" t="str">
-        <v>F1 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="170">
@@ -9389,10 +9450,10 @@
         <v>167</v>
       </c>
       <c r="B170" t="str">
-        <v>HM017</v>
+        <v>HM019</v>
       </c>
       <c r="C170" t="str">
-        <v>Sky sketchers</v>
+        <v>Fifty Shades Of Cache</v>
       </c>
       <c r="D170" t="str">
         <v>Hybrid</v>
@@ -9401,13 +9462,13 @@
         <v>Member 3</v>
       </c>
       <c r="F170" t="str">
-        <v>Undaviya Devarsh Prashant</v>
+        <v>Neev Patel</v>
       </c>
       <c r="G170" t="str">
-        <v>250413101014</v>
+        <v>250410107122</v>
       </c>
       <c r="H170" t="str">
-        <v>9429710151</v>
+        <v>9429400440</v>
       </c>
       <c r="I170" t="str">
         <v/>
@@ -9416,7 +9477,7 @@
         <v/>
       </c>
       <c r="K170" t="str">
-        <v>F1 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="171">
@@ -9424,10 +9485,10 @@
         <v>168</v>
       </c>
       <c r="B171" t="str">
-        <v>HM002</v>
+        <v>HM017</v>
       </c>
       <c r="C171" t="str">
-        <v>Nirmana.io</v>
+        <v>Sky sketchers</v>
       </c>
       <c r="D171" t="str">
         <v>Hybrid</v>
@@ -9436,22 +9497,22 @@
         <v>Team Leader</v>
       </c>
       <c r="F171" t="str">
-        <v>Aum Panchal</v>
+        <v>Patel Aum Dhiren</v>
       </c>
       <c r="G171" t="str">
-        <v>226BEECG001</v>
+        <v>250413101009</v>
       </c>
       <c r="H171" t="str">
-        <v>9157767894</v>
+        <v>8320950668</v>
       </c>
       <c r="I171" t="str">
-        <v>aumpanchal1652007@gmail.com</v>
+        <v>patelaum2266@gmail.com</v>
       </c>
       <c r="J171" t="str">
-        <v>Electronics &amp; Communication (EC)</v>
+        <v>Aeronautical Engineering</v>
       </c>
       <c r="K171" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>F1 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="172">
@@ -9459,10 +9520,10 @@
         <v>169</v>
       </c>
       <c r="B172" t="str">
-        <v>HM002</v>
+        <v>HM017</v>
       </c>
       <c r="C172" t="str">
-        <v>Nirmana.io</v>
+        <v>Sky sketchers</v>
       </c>
       <c r="D172" t="str">
         <v>Hybrid</v>
@@ -9471,13 +9532,13 @@
         <v>Member 1</v>
       </c>
       <c r="F172" t="str">
-        <v>Smit Chaudhari</v>
+        <v>Patel Ayush Saurabh</v>
       </c>
       <c r="G172" t="str">
-        <v>226BEECG002</v>
+        <v>250413101010</v>
       </c>
       <c r="H172" t="str">
-        <v>9157236355</v>
+        <v>9023800699</v>
       </c>
       <c r="I172" t="str">
         <v/>
@@ -9486,7 +9547,7 @@
         <v/>
       </c>
       <c r="K172" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>F1 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="173">
@@ -9494,34 +9555,34 @@
         <v>170</v>
       </c>
       <c r="B173" t="str">
-        <v>HM001</v>
+        <v>HM017</v>
       </c>
       <c r="C173" t="str">
-        <v>Helios</v>
+        <v>Sky sketchers</v>
       </c>
       <c r="D173" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E173" t="str">
-        <v>Team Leader</v>
+        <v>Member 2</v>
       </c>
       <c r="F173" t="str">
-        <v>Jinal Bhavin Mistry</v>
+        <v>Patel Devesh Yogesh</v>
       </c>
       <c r="G173" t="str">
-        <v>26BEECG009</v>
+        <v>250413101002</v>
       </c>
       <c r="H173" t="str">
-        <v>7990849404</v>
+        <v>8160771388</v>
       </c>
       <c r="I173" t="str">
-        <v>12.jinalm@gmail.com</v>
+        <v/>
       </c>
       <c r="J173" t="str">
-        <v>Electronics &amp; Communication (EC)</v>
+        <v/>
       </c>
       <c r="K173" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F1 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="174">
@@ -9529,25 +9590,25 @@
         <v>171</v>
       </c>
       <c r="B174" t="str">
-        <v>HM001</v>
+        <v>HM017</v>
       </c>
       <c r="C174" t="str">
-        <v>Helios</v>
+        <v>Sky sketchers</v>
       </c>
       <c r="D174" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E174" t="str">
-        <v>Member 1</v>
+        <v>Member 3</v>
       </c>
       <c r="F174" t="str">
-        <v>Rishabh Bhagchandani</v>
+        <v>Undaviya Devarsh Prashant</v>
       </c>
       <c r="G174" t="str">
-        <v>26BEECM006</v>
+        <v>250413101014</v>
       </c>
       <c r="H174" t="str">
-        <v>9157391199</v>
+        <v>9429710151</v>
       </c>
       <c r="I174" t="str">
         <v/>
@@ -9556,7 +9617,7 @@
         <v/>
       </c>
       <c r="K174" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F1 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="175">
@@ -9564,34 +9625,34 @@
         <v>172</v>
       </c>
       <c r="B175" t="str">
-        <v>HM001</v>
+        <v>HM002</v>
       </c>
       <c r="C175" t="str">
-        <v>Helios</v>
+        <v>Nirmana.io</v>
       </c>
       <c r="D175" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E175" t="str">
-        <v>Member 2</v>
+        <v>Team Leader</v>
       </c>
       <c r="F175" t="str">
-        <v>Marmik Gandhi</v>
+        <v>Aum Panchal</v>
       </c>
       <c r="G175" t="str">
-        <v>26BEMEM041</v>
+        <v>226BEECG001</v>
       </c>
       <c r="H175" t="str">
-        <v>9265558057</v>
+        <v>9157767894</v>
       </c>
       <c r="I175" t="str">
-        <v/>
+        <v>aumpanchal1652007@gmail.com</v>
       </c>
       <c r="J175" t="str">
-        <v/>
+        <v>Electronics &amp; Communication (EC)</v>
       </c>
       <c r="K175" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="176">
@@ -9599,25 +9660,25 @@
         <v>173</v>
       </c>
       <c r="B176" t="str">
-        <v>HM001</v>
+        <v>HM002</v>
       </c>
       <c r="C176" t="str">
-        <v>Helios</v>
+        <v>Nirmana.io</v>
       </c>
       <c r="D176" t="str">
         <v>Hybrid</v>
       </c>
       <c r="E176" t="str">
-        <v>Member 3</v>
+        <v>Member 1</v>
       </c>
       <c r="F176" t="str">
-        <v>Krishna Thorat</v>
+        <v>Smit Chaudhari</v>
       </c>
       <c r="G176" t="str">
-        <v>26BEECG028</v>
+        <v>226BEECG002</v>
       </c>
       <c r="H176" t="str">
-        <v>9173899957</v>
+        <v>9157236355</v>
       </c>
       <c r="I176" t="str">
         <v/>
@@ -9626,7 +9687,7 @@
         <v/>
       </c>
       <c r="K176" t="str">
-        <v>S4 Lab Second floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="177">
@@ -9634,34 +9695,34 @@
         <v>174</v>
       </c>
       <c r="B177" t="str">
-        <v>XM004</v>
+        <v>HM001</v>
       </c>
       <c r="C177" t="str">
-        <v>FUTURESTACK</v>
+        <v>Helios</v>
       </c>
       <c r="D177" t="str">
-        <v>Hardware</v>
+        <v>Hybrid</v>
       </c>
       <c r="E177" t="str">
         <v>Team Leader</v>
       </c>
       <c r="F177" t="str">
-        <v>PARTH N PRAJAPATI</v>
+        <v>Jinal Bhavin Mistry</v>
       </c>
       <c r="G177" t="str">
-        <v>240410119038</v>
+        <v>26BEECG009</v>
       </c>
       <c r="H177" t="str">
-        <v>9427301801</v>
+        <v>7990849404</v>
       </c>
       <c r="I177" t="str">
-        <v>prajapatiparth2496@gmail.com</v>
+        <v>12.jinalm@gmail.com</v>
       </c>
       <c r="J177" t="str">
-        <v>Mechanical Engineering (ME)</v>
+        <v>Electronics &amp; Communication (EC)</v>
       </c>
       <c r="K177" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="178">
@@ -9669,25 +9730,25 @@
         <v>175</v>
       </c>
       <c r="B178" t="str">
-        <v>XM004</v>
+        <v>HM001</v>
       </c>
       <c r="C178" t="str">
-        <v>FUTURESTACK</v>
+        <v>Helios</v>
       </c>
       <c r="D178" t="str">
-        <v>Hardware</v>
+        <v>Hybrid</v>
       </c>
       <c r="E178" t="str">
         <v>Member 1</v>
       </c>
       <c r="F178" t="str">
-        <v>MUDRA V CHAUHAN</v>
+        <v>Rishabh Bhagchandani</v>
       </c>
       <c r="G178" t="str">
-        <v>240410101005</v>
+        <v>26BEECM006</v>
       </c>
       <c r="H178" t="str">
-        <v>9773119829</v>
+        <v>9157391199</v>
       </c>
       <c r="I178" t="str">
         <v/>
@@ -9696,7 +9757,7 @@
         <v/>
       </c>
       <c r="K178" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="179">
@@ -9704,25 +9765,25 @@
         <v>176</v>
       </c>
       <c r="B179" t="str">
-        <v>XM004</v>
+        <v>HM001</v>
       </c>
       <c r="C179" t="str">
-        <v>FUTURESTACK</v>
+        <v>Helios</v>
       </c>
       <c r="D179" t="str">
-        <v>Hardware</v>
+        <v>Hybrid</v>
       </c>
       <c r="E179" t="str">
         <v>Member 2</v>
       </c>
       <c r="F179" t="str">
-        <v>HARSHIL PANCHAL</v>
+        <v>Marmik Gandhi</v>
       </c>
       <c r="G179" t="str">
-        <v>240410119023</v>
+        <v>26BEMEM041</v>
       </c>
       <c r="H179" t="str">
-        <v>9974988786</v>
+        <v>9265558057</v>
       </c>
       <c r="I179" t="str">
         <v/>
@@ -9731,7 +9792,7 @@
         <v/>
       </c>
       <c r="K179" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="180">
@@ -9739,25 +9800,25 @@
         <v>177</v>
       </c>
       <c r="B180" t="str">
-        <v>XM004</v>
+        <v>HM001</v>
       </c>
       <c r="C180" t="str">
-        <v>FUTURESTACK</v>
+        <v>Helios</v>
       </c>
       <c r="D180" t="str">
-        <v>Hardware</v>
+        <v>Hybrid</v>
       </c>
       <c r="E180" t="str">
         <v>Member 3</v>
       </c>
       <c r="F180" t="str">
-        <v>HARDEEP BHAVSAR</v>
+        <v>Krishna Thorat</v>
       </c>
       <c r="G180" t="str">
-        <v>240410119009</v>
+        <v>26BEECG028</v>
       </c>
       <c r="H180" t="str">
-        <v>9510945029</v>
+        <v>9173899957</v>
       </c>
       <c r="I180" t="str">
         <v/>
@@ -9766,7 +9827,7 @@
         <v/>
       </c>
       <c r="K180" t="str">
-        <v>F4 Lab First floor CE dept.</v>
+        <v>S4 Lab Second floor CE dept.</v>
       </c>
     </row>
     <row r="181">
@@ -9774,10 +9835,10 @@
         <v>178</v>
       </c>
       <c r="B181" t="str">
-        <v>XM001</v>
+        <v>XM004</v>
       </c>
       <c r="C181" t="str">
-        <v>NextLift</v>
+        <v>FUTURESTACK</v>
       </c>
       <c r="D181" t="str">
         <v>Hardware</v>
@@ -9786,22 +9847,22 @@
         <v>Team Leader</v>
       </c>
       <c r="F181" t="str">
-        <v>Shah Prayag Bhaveshbhai</v>
+        <v>PARTH N PRAJAPATI</v>
       </c>
       <c r="G181" t="str">
-        <v>240410101049</v>
+        <v>240410119038</v>
       </c>
       <c r="H181" t="str">
-        <v>8200088416</v>
+        <v>9427301801</v>
       </c>
       <c r="I181" t="str">
-        <v>prayag1602@gmail.com</v>
+        <v>prajapatiparth2496@gmail.com</v>
       </c>
       <c r="J181" t="str">
-        <v>Aeronautical Engineering</v>
+        <v>Mechanical Engineering (ME)</v>
       </c>
       <c r="K181" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="182">
@@ -9809,10 +9870,10 @@
         <v>179</v>
       </c>
       <c r="B182" t="str">
-        <v>XM001</v>
+        <v>XM004</v>
       </c>
       <c r="C182" t="str">
-        <v>NextLift</v>
+        <v>FUTURESTACK</v>
       </c>
       <c r="D182" t="str">
         <v>Hardware</v>
@@ -9821,13 +9882,13 @@
         <v>Member 1</v>
       </c>
       <c r="F182" t="str">
-        <v>Solanki Mudra Vishalkumar</v>
+        <v>MUDRA V CHAUHAN</v>
       </c>
       <c r="G182" t="str">
-        <v>240410101028</v>
+        <v>240410101005</v>
       </c>
       <c r="H182" t="str">
-        <v>7990580277</v>
+        <v>9773119829</v>
       </c>
       <c r="I182" t="str">
         <v/>
@@ -9836,7 +9897,7 @@
         <v/>
       </c>
       <c r="K182" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="183">
@@ -9844,10 +9905,10 @@
         <v>180</v>
       </c>
       <c r="B183" t="str">
-        <v>XM001</v>
+        <v>XM004</v>
       </c>
       <c r="C183" t="str">
-        <v>NextLift</v>
+        <v>FUTURESTACK</v>
       </c>
       <c r="D183" t="str">
         <v>Hardware</v>
@@ -9856,13 +9917,13 @@
         <v>Member 2</v>
       </c>
       <c r="F183" t="str">
-        <v>Vasava Hetvi Subhashbhai</v>
+        <v>HARSHIL PANCHAL</v>
       </c>
       <c r="G183" t="str">
-        <v>240410101062</v>
+        <v>240410119023</v>
       </c>
       <c r="H183" t="str">
-        <v>8459451983</v>
+        <v>9974988786</v>
       </c>
       <c r="I183" t="str">
         <v/>
@@ -9871,7 +9932,7 @@
         <v/>
       </c>
       <c r="K183" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="184">
@@ -9879,10 +9940,10 @@
         <v>181</v>
       </c>
       <c r="B184" t="str">
-        <v>XM001</v>
+        <v>XM004</v>
       </c>
       <c r="C184" t="str">
-        <v>NextLift</v>
+        <v>FUTURESTACK</v>
       </c>
       <c r="D184" t="str">
         <v>Hardware</v>
@@ -9891,13 +9952,13 @@
         <v>Member 3</v>
       </c>
       <c r="F184" t="str">
-        <v>Patel Vishva Nileshkumar</v>
+        <v>HARDEEP BHAVSAR</v>
       </c>
       <c r="G184" t="str">
-        <v>240410107205</v>
+        <v>240410119009</v>
       </c>
       <c r="H184" t="str">
-        <v>9173715752</v>
+        <v>9510945029</v>
       </c>
       <c r="I184" t="str">
         <v/>
@@ -9906,7 +9967,7 @@
         <v/>
       </c>
       <c r="K184" t="str">
-        <v>F5 Lab First floor CE dept.</v>
+        <v>F4 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="185">
@@ -9914,10 +9975,10 @@
         <v>182</v>
       </c>
       <c r="B185" t="str">
-        <v>XM005</v>
+        <v>XM001</v>
       </c>
       <c r="C185" t="str">
-        <v>VoltForage</v>
+        <v>NextLift</v>
       </c>
       <c r="D185" t="str">
         <v>Hardware</v>
@@ -9926,22 +9987,22 @@
         <v>Team Leader</v>
       </c>
       <c r="F185" t="str">
-        <v>Shubh Prajapati</v>
+        <v>Shah Prayag Bhaveshbhai</v>
       </c>
       <c r="G185" t="str">
-        <v>250410111023</v>
+        <v>240410101049</v>
       </c>
       <c r="H185" t="str">
-        <v>9601983862</v>
+        <v>8200088416</v>
       </c>
       <c r="I185" t="str">
-        <v>shubhatwork555@gmail.com</v>
+        <v>prayag1602@gmail.com</v>
       </c>
       <c r="J185" t="str">
-        <v>Electronics &amp; Communication (EC)</v>
+        <v>Aeronautical Engineering</v>
       </c>
       <c r="K185" t="str">
-        <v>G3 Lab Ground floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="186">
@@ -9949,10 +10010,10 @@
         <v>183</v>
       </c>
       <c r="B186" t="str">
-        <v>XM005</v>
+        <v>XM001</v>
       </c>
       <c r="C186" t="str">
-        <v>VoltForage</v>
+        <v>NextLift</v>
       </c>
       <c r="D186" t="str">
         <v>Hardware</v>
@@ -9961,13 +10022,13 @@
         <v>Member 1</v>
       </c>
       <c r="F186" t="str">
-        <v>Tejas Soni</v>
+        <v>Solanki Mudra Vishalkumar</v>
       </c>
       <c r="G186" t="str">
-        <v>250410111031</v>
+        <v>240410101028</v>
       </c>
       <c r="H186" t="str">
-        <v>9574042008</v>
+        <v>7990580277</v>
       </c>
       <c r="I186" t="str">
         <v/>
@@ -9976,7 +10037,7 @@
         <v/>
       </c>
       <c r="K186" t="str">
-        <v>G3 Lab Ground floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="187">
@@ -9984,10 +10045,10 @@
         <v>184</v>
       </c>
       <c r="B187" t="str">
-        <v>XM005</v>
+        <v>XM001</v>
       </c>
       <c r="C187" t="str">
-        <v>VoltForage</v>
+        <v>NextLift</v>
       </c>
       <c r="D187" t="str">
         <v>Hardware</v>
@@ -9996,13 +10057,13 @@
         <v>Member 2</v>
       </c>
       <c r="F187" t="str">
-        <v>Vraj Prajapati</v>
+        <v>Vasava Hetvi Subhashbhai</v>
       </c>
       <c r="G187" t="str">
-        <v>250410111024</v>
+        <v>240410101062</v>
       </c>
       <c r="H187" t="str">
-        <v>7861041755</v>
+        <v>8459451983</v>
       </c>
       <c r="I187" t="str">
         <v/>
@@ -10011,7 +10072,7 @@
         <v/>
       </c>
       <c r="K187" t="str">
-        <v>G3 Lab Ground floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="188">
@@ -10019,10 +10080,10 @@
         <v>185</v>
       </c>
       <c r="B188" t="str">
-        <v>XM005</v>
+        <v>XM001</v>
       </c>
       <c r="C188" t="str">
-        <v>VoltForage</v>
+        <v>NextLift</v>
       </c>
       <c r="D188" t="str">
         <v>Hardware</v>
@@ -10031,13 +10092,13 @@
         <v>Member 3</v>
       </c>
       <c r="F188" t="str">
-        <v>Vaishnavi S</v>
+        <v>Patel Vishva Nileshkumar</v>
       </c>
       <c r="G188" t="str">
-        <v>250410111027</v>
+        <v>240410107205</v>
       </c>
       <c r="H188" t="str">
-        <v>8866885465</v>
+        <v>9173715752</v>
       </c>
       <c r="I188" t="str">
         <v/>
@@ -10046,7 +10107,7 @@
         <v/>
       </c>
       <c r="K188" t="str">
-        <v>G3 Lab Ground floor CE dept.</v>
+        <v>F5 Lab First floor CE dept.</v>
       </c>
     </row>
     <row r="189">
@@ -10054,10 +10115,10 @@
         <v>186</v>
       </c>
       <c r="B189" t="str">
-        <v>XM002</v>
+        <v>XM005</v>
       </c>
       <c r="C189" t="str">
-        <v>Akatsuki</v>
+        <v>VoltForage</v>
       </c>
       <c r="D189" t="str">
         <v>Hardware</v>
@@ -10066,19 +10127,19 @@
         <v>Team Leader</v>
       </c>
       <c r="F189" t="str">
-        <v>Harnish Yogesh More</v>
+        <v>Shubh Prajapati</v>
       </c>
       <c r="G189" t="str">
-        <v>240410109002/24BEEEG011</v>
+        <v>250410111023</v>
       </c>
       <c r="H189" t="str">
-        <v>7405324209</v>
+        <v>9601983862</v>
       </c>
       <c r="I189" t="str">
-        <v>harnishmore2006@gmail.com</v>
+        <v>shubhatwork555@gmail.com</v>
       </c>
       <c r="J189" t="str">
-        <v>Electrical Engineering (EE)</v>
+        <v>Electronics &amp; Communication (EC)</v>
       </c>
       <c r="K189" t="str">
         <v>G3 Lab Ground floor CE dept.</v>
@@ -10089,10 +10150,10 @@
         <v>187</v>
       </c>
       <c r="B190" t="str">
-        <v>XM002</v>
+        <v>XM005</v>
       </c>
       <c r="C190" t="str">
-        <v>Akatsuki</v>
+        <v>VoltForage</v>
       </c>
       <c r="D190" t="str">
         <v>Hardware</v>
@@ -10101,13 +10162,13 @@
         <v>Member 1</v>
       </c>
       <c r="F190" t="str">
-        <v>Tirth Parmar</v>
+        <v>Tejas Soni</v>
       </c>
       <c r="G190" t="str">
-        <v>240410109008</v>
+        <v>250410111031</v>
       </c>
       <c r="H190" t="str">
-        <v>9016862388</v>
+        <v>9574042008</v>
       </c>
       <c r="I190" t="str">
         <v/>
@@ -10124,10 +10185,10 @@
         <v>188</v>
       </c>
       <c r="B191" t="str">
-        <v>XM002</v>
+        <v>XM005</v>
       </c>
       <c r="C191" t="str">
-        <v>Akatsuki</v>
+        <v>VoltForage</v>
       </c>
       <c r="D191" t="str">
         <v>Hardware</v>
@@ -10136,13 +10197,13 @@
         <v>Member 2</v>
       </c>
       <c r="F191" t="str">
-        <v>Aditya Soni</v>
+        <v>Vraj Prajapati</v>
       </c>
       <c r="G191" t="str">
-        <v>250413109015</v>
+        <v>250410111024</v>
       </c>
       <c r="H191" t="str">
-        <v>7434926341</v>
+        <v>7861041755</v>
       </c>
       <c r="I191" t="str">
         <v/>
@@ -10159,10 +10220,10 @@
         <v>189</v>
       </c>
       <c r="B192" t="str">
-        <v>XM002</v>
+        <v>XM005</v>
       </c>
       <c r="C192" t="str">
-        <v>Akatsuki</v>
+        <v>VoltForage</v>
       </c>
       <c r="D192" t="str">
         <v>Hardware</v>
@@ -10171,13 +10232,13 @@
         <v>Member 3</v>
       </c>
       <c r="F192" t="str">
-        <v>Viraj Kalekar</v>
+        <v>Vaishnavi S</v>
       </c>
       <c r="G192" t="str">
-        <v>240410109003</v>
+        <v>250410111027</v>
       </c>
       <c r="H192" t="str">
-        <v>9558991947</v>
+        <v>8866885465</v>
       </c>
       <c r="I192" t="str">
         <v/>
@@ -10189,16 +10250,156 @@
         <v>G3 Lab Ground floor CE dept.</v>
       </c>
     </row>
+    <row r="193">
+      <c r="A193">
+        <v>190</v>
+      </c>
+      <c r="B193" t="str">
+        <v>XM002</v>
+      </c>
+      <c r="C193" t="str">
+        <v>Akatsuki</v>
+      </c>
+      <c r="D193" t="str">
+        <v>Hardware</v>
+      </c>
+      <c r="E193" t="str">
+        <v>Team Leader</v>
+      </c>
+      <c r="F193" t="str">
+        <v>Harnish Yogesh More</v>
+      </c>
+      <c r="G193" t="str">
+        <v>240410109002/24BEEEG011</v>
+      </c>
+      <c r="H193" t="str">
+        <v>7405324209</v>
+      </c>
+      <c r="I193" t="str">
+        <v>harnishmore2006@gmail.com</v>
+      </c>
+      <c r="J193" t="str">
+        <v>Electrical Engineering (EE)</v>
+      </c>
+      <c r="K193" t="str">
+        <v>G3 Lab Ground floor CE dept.</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194">
+        <v>191</v>
+      </c>
+      <c r="B194" t="str">
+        <v>XM002</v>
+      </c>
+      <c r="C194" t="str">
+        <v>Akatsuki</v>
+      </c>
+      <c r="D194" t="str">
+        <v>Hardware</v>
+      </c>
+      <c r="E194" t="str">
+        <v>Member 1</v>
+      </c>
+      <c r="F194" t="str">
+        <v>Tirth Parmar</v>
+      </c>
+      <c r="G194" t="str">
+        <v>240410109008</v>
+      </c>
+      <c r="H194" t="str">
+        <v>9016862388</v>
+      </c>
+      <c r="I194" t="str">
+        <v/>
+      </c>
+      <c r="J194" t="str">
+        <v/>
+      </c>
+      <c r="K194" t="str">
+        <v>G3 Lab Ground floor CE dept.</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195">
+        <v>192</v>
+      </c>
+      <c r="B195" t="str">
+        <v>XM002</v>
+      </c>
+      <c r="C195" t="str">
+        <v>Akatsuki</v>
+      </c>
+      <c r="D195" t="str">
+        <v>Hardware</v>
+      </c>
+      <c r="E195" t="str">
+        <v>Member 2</v>
+      </c>
+      <c r="F195" t="str">
+        <v>Aditya Soni</v>
+      </c>
+      <c r="G195" t="str">
+        <v>250413109015</v>
+      </c>
+      <c r="H195" t="str">
+        <v>7434926341</v>
+      </c>
+      <c r="I195" t="str">
+        <v/>
+      </c>
+      <c r="J195" t="str">
+        <v/>
+      </c>
+      <c r="K195" t="str">
+        <v>G3 Lab Ground floor CE dept.</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196">
+        <v>193</v>
+      </c>
+      <c r="B196" t="str">
+        <v>XM002</v>
+      </c>
+      <c r="C196" t="str">
+        <v>Akatsuki</v>
+      </c>
+      <c r="D196" t="str">
+        <v>Hardware</v>
+      </c>
+      <c r="E196" t="str">
+        <v>Member 3</v>
+      </c>
+      <c r="F196" t="str">
+        <v>Viraj Kalekar</v>
+      </c>
+      <c r="G196" t="str">
+        <v>240410109003</v>
+      </c>
+      <c r="H196" t="str">
+        <v>9558991947</v>
+      </c>
+      <c r="I196" t="str">
+        <v/>
+      </c>
+      <c r="J196" t="str">
+        <v/>
+      </c>
+      <c r="K196" t="str">
+        <v>G3 Lab Ground floor CE dept.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K192"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K196"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J34"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10214,7 +10415,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>MECIA HACKS 3.0 — SOFTWARE TRACK FINALISTS (30 TEAMS)</v>
+        <v>MECIA HACKS 3.0 — SOFTWARE TRACK FINALISTS (31 TEAMS)</v>
       </c>
     </row>
     <row r="3">
@@ -11209,9 +11410,41 @@
         <v>G3 Lab Ground floor CE dept.</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34">
+        <v>31</v>
+      </c>
+      <c r="B34" t="str">
+        <v>SM065</v>
+      </c>
+      <c r="C34" t="str">
+        <v>A.S.T.R.A</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Aryan Mohite</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Aditya Mathur, Anshul Chainani, Ishit Bhavsar</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Aditya Mathur</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Anshul Chainani</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Ishit Bhavsar</v>
+      </c>
+      <c r="I34" t="str">
+        <v>S.A.D.H.A.K</v>
+      </c>
+      <c r="J34" t="str">
+        <v>F4 Lab First floor CE dept.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J34"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>